<commit_message>
Lưu tiến độ trước khi thêm thẩm định Phụ lục I.5
Bao gồm lưu trữ SQLite, quản lý đơn vị 4 cấp, launcher session,
xuất báo cáo RAW theo mẫu BQP (chỉ I, I.1-I.5, tổng hợp cấp 2 khi xuất cấp 1)
và sửa định dạng số tiền ô hai dòng khi xuất thẩm định.

Không đưa 2 file dữ liệu nhân sự BTL Hà Nội vào repo (repo công khai).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/main/resources/static/26.9.PHU_LUC_SUA.xlsx
+++ b/src/main/resources/static/26.9.PHU_LUC_SUA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\bqp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B8DD64-6BF2-42AE-8534-372A1AA30801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA1E8CFD-AD42-4F8C-BB34-3B1299E59CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="19128" windowHeight="16800" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16920" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Phụ lục I" sheetId="5" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="209">
   <si>
     <t>Số TT</t>
   </si>
@@ -463,27 +463,6 @@
     </r>
   </si>
   <si>
-    <t>12= cột 10*(0,8 * cột 9)</t>
-  </si>
-  <si>
-    <t>13= cột 11*(1,5* cột 9)</t>
-  </si>
-  <si>
-    <t>14= 3*cột 9</t>
-  </si>
-  <si>
-    <t>15= cột 10*(0,4* cột 9)</t>
-  </si>
-  <si>
-    <t>16= cột 11*(1,5*cột 9)</t>
-  </si>
-  <si>
-    <t>17= 3*cột 9</t>
-  </si>
-  <si>
-    <t>18= cột 12 đến cột 17</t>
-  </si>
-  <si>
     <t>TỔNG HỢP KINH PHÍ CHI TRẢ CHẾ ĐỘ NGHỊ ĐỊNH SỐ 178/2024/NĐ-CP</t>
   </si>
   <si>
@@ -512,24 +491,6 @@
   </si>
   <si>
     <t>Số năm nghỉ sớm hưởng trợ cấp theo Hướng dẫn số 1787/HD-BQP</t>
-  </si>
-  <si>
-    <t>10 = Cột 8 - Cột 5</t>
-  </si>
-  <si>
-    <t>14= Cột 9*0,5 tháng (Cột 10-20 (15) năm)</t>
-  </si>
-  <si>
-    <t>15= Cột 12 đến Cột 14</t>
-  </si>
-  <si>
-    <t>13= Cột 9*5 tháng (Cột 10&gt;20 năm hoặc &gt;15)</t>
-  </si>
-  <si>
-    <t>11= (trần quân hàm + Cột 2) - Cột 8</t>
-  </si>
-  <si>
-    <t>12= Cột 11*(5 tháng* Cột 9)</t>
   </si>
   <si>
     <t>Biên chế</t>
@@ -949,6 +910,27 @@
       </rPr>
       <t xml:space="preserve"> (chức vụ tại thời điểm hưởng chế độ)</t>
     </r>
+  </si>
+  <si>
+    <t>4//</t>
+  </si>
+  <si>
+    <t>Trợ lý</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3/1988</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 7/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2/1970</t>
+  </si>
+  <si>
+    <t>ĐV</t>
   </si>
 </sst>
 </file>
@@ -1753,24 +1735,66 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1793,7 +1817,14 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1806,19 +1837,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1859,33 +1881,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1893,41 +1890,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -2233,36 +2213,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="131" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="107" t="s">
-        <v>134</v>
-      </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="110" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
     </row>
     <row r="2" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="109" t="s">
+      <c r="A2" s="132" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="109"/>
-      <c r="C2" s="110" t="s">
-        <v>183</v>
-      </c>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
-      <c r="F2" s="110"/>
-      <c r="G2" s="110"/>
-      <c r="H2" s="110"/>
-      <c r="I2" s="110"/>
-      <c r="J2" s="110"/>
+      <c r="B2" s="132"/>
+      <c r="C2" s="133" t="s">
+        <v>170</v>
+      </c>
+      <c r="D2" s="133"/>
+      <c r="E2" s="133"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="133"/>
+      <c r="H2" s="133"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="133"/>
       <c r="L2" s="74"/>
       <c r="M2" s="30"/>
       <c r="N2" s="30"/>
@@ -2274,16 +2254,16 @@
     </row>
     <row r="3" spans="1:21" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="20"/>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115"/>
       <c r="K3" s="20"/>
       <c r="L3" s="20"/>
       <c r="M3" s="20"/>
@@ -2304,11 +2284,11 @@
       <c r="E4" s="32"/>
       <c r="F4" s="30"/>
       <c r="G4" s="32"/>
-      <c r="H4" s="99" t="s">
-        <v>111</v>
-      </c>
-      <c r="I4" s="99"/>
-      <c r="J4" s="99"/>
+      <c r="H4" s="119" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="119"/>
+      <c r="J4" s="119"/>
       <c r="K4" s="30"/>
       <c r="L4" s="30"/>
       <c r="M4" s="30"/>
@@ -2320,28 +2300,28 @@
       <c r="S4" s="30"/>
     </row>
     <row r="5" spans="1:21" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="100" t="s">
-        <v>112</v>
-      </c>
-      <c r="B5" s="102" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="103" t="s">
-        <v>197</v>
-      </c>
-      <c r="D5" s="104"/>
-      <c r="E5" s="103" t="s">
-        <v>198</v>
-      </c>
-      <c r="F5" s="104"/>
-      <c r="G5" s="103" t="s">
-        <v>199</v>
-      </c>
-      <c r="H5" s="105"/>
-      <c r="I5" s="103" t="s">
+      <c r="A5" s="120" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="122" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="123" t="s">
+        <v>184</v>
+      </c>
+      <c r="D5" s="124"/>
+      <c r="E5" s="123" t="s">
+        <v>185</v>
+      </c>
+      <c r="F5" s="124"/>
+      <c r="G5" s="123" t="s">
+        <v>186</v>
+      </c>
+      <c r="H5" s="125"/>
+      <c r="I5" s="123" t="s">
         <v>67</v>
       </c>
-      <c r="J5" s="106"/>
+      <c r="J5" s="126"/>
       <c r="K5" s="30"/>
       <c r="L5" s="30"/>
       <c r="M5" s="30"/>
@@ -2353,8 +2333,8 @@
       <c r="S5" s="30"/>
     </row>
     <row r="6" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="101"/>
-      <c r="B6" s="101"/>
+      <c r="A6" s="121"/>
+      <c r="B6" s="121"/>
       <c r="C6" s="33" t="s">
         <v>56</v>
       </c>
@@ -2415,10 +2395,10 @@
         <v>6</v>
       </c>
       <c r="I7" s="35" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="J7" s="35" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="K7" s="36"/>
       <c r="L7" s="36"/>
@@ -2435,7 +2415,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="39" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="C8" s="40"/>
       <c r="D8" s="41"/>
@@ -2460,7 +2440,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="39" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="C9" s="46"/>
       <c r="D9" s="47"/>
@@ -2485,7 +2465,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="C10" s="46"/>
       <c r="D10" s="47"/>
@@ -2510,7 +2490,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="C11" s="46"/>
       <c r="D11" s="47"/>
@@ -2535,7 +2515,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="C12" s="49"/>
       <c r="D12" s="50"/>
@@ -2560,7 +2540,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="C13" s="46"/>
       <c r="D13" s="47"/>
@@ -2585,7 +2565,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="39" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="C14" s="46"/>
       <c r="D14" s="47"/>
@@ -2610,7 +2590,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="C15" s="46"/>
       <c r="D15" s="47"/>
@@ -2635,7 +2615,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>192</v>
+        <v>179</v>
       </c>
       <c r="C16" s="46"/>
       <c r="D16" s="47"/>
@@ -2700,18 +2680,18 @@
       <c r="S18" s="30"/>
     </row>
     <row r="19" spans="1:19" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="94" t="s">
-        <v>193</v>
-      </c>
-      <c r="B19" s="94"/>
-      <c r="C19" s="94"/>
-      <c r="D19" s="94"/>
-      <c r="E19" s="94"/>
-      <c r="F19" s="94"/>
-      <c r="G19" s="94"/>
-      <c r="H19" s="94"/>
-      <c r="I19" s="94"/>
-      <c r="J19" s="94"/>
+      <c r="A19" s="127" t="s">
+        <v>180</v>
+      </c>
+      <c r="B19" s="127"/>
+      <c r="C19" s="127"/>
+      <c r="D19" s="127"/>
+      <c r="E19" s="127"/>
+      <c r="F19" s="127"/>
+      <c r="G19" s="127"/>
+      <c r="H19" s="127"/>
+      <c r="I19" s="127"/>
+      <c r="J19" s="127"/>
       <c r="K19" s="72"/>
       <c r="L19" s="72"/>
       <c r="M19" s="72"/>
@@ -2730,9 +2710,9 @@
       <c r="E20" s="73"/>
       <c r="F20" s="72"/>
       <c r="G20" s="73"/>
-      <c r="H20" s="95"/>
-      <c r="I20" s="95"/>
-      <c r="J20" s="96"/>
+      <c r="H20" s="128"/>
+      <c r="I20" s="128"/>
+      <c r="J20" s="129"/>
       <c r="K20" s="72"/>
       <c r="L20" s="72"/>
       <c r="M20" s="72"/>
@@ -2745,14 +2725,14 @@
     </row>
     <row r="21" spans="1:19" ht="13.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="22"/>
-      <c r="C21" s="97"/>
-      <c r="D21" s="96"/>
-      <c r="E21" s="96"/>
-      <c r="F21" s="96"/>
-      <c r="G21" s="96"/>
-      <c r="H21" s="97"/>
-      <c r="I21" s="97"/>
-      <c r="J21" s="96"/>
+      <c r="C21" s="130"/>
+      <c r="D21" s="129"/>
+      <c r="E21" s="129"/>
+      <c r="F21" s="129"/>
+      <c r="G21" s="129"/>
+      <c r="H21" s="130"/>
+      <c r="I21" s="130"/>
+      <c r="J21" s="129"/>
       <c r="K21" s="22"/>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -2871,14 +2851,14 @@
     <row r="27" spans="1:19" s="75" customFormat="1" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="29"/>
       <c r="B27" s="29"/>
-      <c r="C27" s="98"/>
-      <c r="D27" s="98"/>
-      <c r="E27" s="98"/>
-      <c r="F27" s="98"/>
-      <c r="G27" s="98"/>
-      <c r="H27" s="98"/>
-      <c r="I27" s="98"/>
-      <c r="J27" s="98"/>
+      <c r="C27" s="118"/>
+      <c r="D27" s="118"/>
+      <c r="E27" s="118"/>
+      <c r="F27" s="118"/>
+      <c r="G27" s="118"/>
+      <c r="H27" s="118"/>
+      <c r="I27" s="118"/>
+      <c r="J27" s="118"/>
       <c r="K27" s="74"/>
       <c r="L27" s="74"/>
       <c r="M27" s="74"/>
@@ -23202,6 +23182,7 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="C27:G27"/>
     <mergeCell ref="H27:J27"/>
     <mergeCell ref="H4:J4"/>
@@ -23211,7 +23192,6 @@
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="I5:J5"/>
-    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A19:J19"/>
     <mergeCell ref="H20:J20"/>
     <mergeCell ref="C21:G21"/>
@@ -23233,90 +23213,94 @@
   <cols>
     <col min="1" max="1" width="3.69921875" customWidth="1"/>
     <col min="2" max="2" width="21.296875" customWidth="1"/>
+    <col min="9" max="9" width="9.8984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.8984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="19" width="10.8984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="110" t="s">
         <v>63</v>
       </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="107"/>
-      <c r="O1" s="107"/>
-      <c r="P1" s="107"/>
-      <c r="Q1" s="107"/>
-      <c r="R1" s="107"/>
-      <c r="S1" s="107"/>
-      <c r="T1" s="107"/>
-      <c r="U1" s="107"/>
-      <c r="V1" s="107"/>
-      <c r="W1" s="107"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="110"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="110"/>
+      <c r="S1" s="110"/>
+      <c r="T1" s="110"/>
+      <c r="U1" s="110"/>
+      <c r="V1" s="110"/>
+      <c r="W1" s="110"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="107" t="s">
-        <v>196</v>
-      </c>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
-      <c r="M2" s="107"/>
-      <c r="N2" s="107"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="107"/>
-      <c r="Q2" s="107"/>
-      <c r="R2" s="107"/>
-      <c r="S2" s="107"/>
-      <c r="T2" s="107"/>
-      <c r="U2" s="107"/>
-      <c r="V2" s="107"/>
-      <c r="W2" s="107"/>
+      <c r="C2" s="110" t="s">
+        <v>183</v>
+      </c>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
+      <c r="L2" s="110"/>
+      <c r="M2" s="110"/>
+      <c r="N2" s="110"/>
+      <c r="O2" s="110"/>
+      <c r="P2" s="110"/>
+      <c r="Q2" s="110"/>
+      <c r="R2" s="110"/>
+      <c r="S2" s="110"/>
+      <c r="T2" s="110"/>
+      <c r="U2" s="110"/>
+      <c r="V2" s="110"/>
+      <c r="W2" s="110"/>
     </row>
     <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.35">
       <c r="B3" s="3"/>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
-      <c r="P3" s="93"/>
-      <c r="Q3" s="93"/>
-      <c r="R3" s="93"/>
-      <c r="S3" s="93"/>
-      <c r="T3" s="93"/>
-      <c r="U3" s="93"/>
-      <c r="V3" s="93"/>
-      <c r="W3" s="93"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115"/>
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="115"/>
+      <c r="S3" s="115"/>
+      <c r="T3" s="115"/>
+      <c r="U3" s="115"/>
+      <c r="V3" s="115"/>
+      <c r="W3" s="115"/>
     </row>
     <row r="4" spans="1:23" s="15" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="C4" s="16"/>
@@ -23336,106 +23320,106 @@
       <c r="W5" s="21"/>
     </row>
     <row r="6" spans="1:23" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="91" t="s">
+      <c r="A6" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="91" t="s">
+      <c r="B6" s="111" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="91" t="s">
+      <c r="C6" s="111" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="91" t="s">
+      <c r="D6" s="111" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="91" t="s">
+      <c r="E6" s="111" t="s">
         <v>102</v>
       </c>
-      <c r="F6" s="91" t="s">
+      <c r="F6" s="111" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="91" t="s">
+      <c r="H6" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="91" t="s">
+      <c r="I6" s="111" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="91" t="s">
+      <c r="J6" s="111" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="91" t="s">
+      <c r="K6" s="111" t="s">
         <v>53</v>
       </c>
-      <c r="L6" s="91" t="s">
+      <c r="L6" s="111" t="s">
         <v>55</v>
       </c>
-      <c r="M6" s="91" t="s">
+      <c r="M6" s="111" t="s">
         <v>13</v>
       </c>
-      <c r="N6" s="91"/>
-      <c r="O6" s="91"/>
-      <c r="P6" s="91"/>
-      <c r="Q6" s="113" t="s">
+      <c r="N6" s="111"/>
+      <c r="O6" s="111"/>
+      <c r="P6" s="111"/>
+      <c r="Q6" s="112" t="s">
         <v>16</v>
       </c>
-      <c r="R6" s="114"/>
-      <c r="S6" s="114"/>
-      <c r="T6" s="114"/>
-      <c r="U6" s="114"/>
-      <c r="V6" s="115"/>
-      <c r="W6" s="91" t="s">
+      <c r="R6" s="113"/>
+      <c r="S6" s="113"/>
+      <c r="T6" s="113"/>
+      <c r="U6" s="113"/>
+      <c r="V6" s="114"/>
+      <c r="W6" s="111" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:23" s="1" customFormat="1" ht="61.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="91"/>
-      <c r="B7" s="91"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="91"/>
-      <c r="K7" s="91"/>
-      <c r="L7" s="91"/>
-      <c r="M7" s="91" t="s">
+      <c r="A7" s="111"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="111"/>
+      <c r="E7" s="111"/>
+      <c r="F7" s="111"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="111"/>
+      <c r="I7" s="111"/>
+      <c r="J7" s="111"/>
+      <c r="K7" s="111"/>
+      <c r="L7" s="111"/>
+      <c r="M7" s="111" t="s">
         <v>9</v>
       </c>
-      <c r="N7" s="91"/>
-      <c r="O7" s="91" t="s">
+      <c r="N7" s="111"/>
+      <c r="O7" s="111" t="s">
         <v>12</v>
       </c>
-      <c r="P7" s="91"/>
-      <c r="Q7" s="91" t="s">
+      <c r="P7" s="111"/>
+      <c r="Q7" s="111" t="s">
         <v>14</v>
       </c>
-      <c r="R7" s="91"/>
-      <c r="S7" s="91"/>
-      <c r="T7" s="91" t="s">
+      <c r="R7" s="111"/>
+      <c r="S7" s="111"/>
+      <c r="T7" s="111" t="s">
         <v>15</v>
       </c>
-      <c r="U7" s="91"/>
-      <c r="V7" s="91"/>
-      <c r="W7" s="91"/>
-    </row>
-    <row r="8" spans="1:23" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="91"/>
-      <c r="B8" s="91"/>
-      <c r="C8" s="91"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
-      <c r="K8" s="91"/>
-      <c r="L8" s="91"/>
+      <c r="U7" s="111"/>
+      <c r="V7" s="111"/>
+      <c r="W7" s="111"/>
+    </row>
+    <row r="8" spans="1:23" ht="156" x14ac:dyDescent="0.3">
+      <c r="A8" s="111"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="111"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="111"/>
+      <c r="G8" s="111"/>
+      <c r="H8" s="111"/>
+      <c r="I8" s="111"/>
+      <c r="J8" s="111"/>
+      <c r="K8" s="111"/>
+      <c r="L8" s="111"/>
       <c r="M8" s="7" t="s">
         <v>10</v>
       </c>
@@ -23466,9 +23450,9 @@
       <c r="V8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="W8" s="91"/>
-    </row>
-    <row r="9" spans="1:23" s="10" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="W8" s="111"/>
+    </row>
+    <row r="9" spans="1:23" s="10" customFormat="1" ht="10.199999999999999" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>1</v>
       </c>
@@ -23505,44 +23489,46 @@
       <c r="L9" s="9">
         <v>12</v>
       </c>
-      <c r="M9" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="N9" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="O9" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="P9" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q9" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="R9" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="S9" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="T9" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="U9" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="V9" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="W9" s="9" t="s">
-        <v>35</v>
+      <c r="M9" s="9">
+        <v>13</v>
+      </c>
+      <c r="N9" s="9">
+        <v>14</v>
+      </c>
+      <c r="O9" s="9">
+        <v>15</v>
+      </c>
+      <c r="P9" s="9">
+        <v>16</v>
+      </c>
+      <c r="Q9" s="9">
+        <v>17</v>
+      </c>
+      <c r="R9" s="9">
+        <v>18</v>
+      </c>
+      <c r="S9" s="9">
+        <v>19</v>
+      </c>
+      <c r="T9" s="9">
+        <v>20</v>
+      </c>
+      <c r="U9" s="9">
+        <v>21</v>
+      </c>
+      <c r="V9" s="9">
+        <v>22</v>
+      </c>
+      <c r="W9" s="9">
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:23" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
+      <c r="A10" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B10" s="14" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -23602,27 +23588,57 @@
       <c r="B12" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
+      <c r="C12" s="107" t="s">
+        <v>207</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="F12" s="107" t="s">
+        <v>204</v>
+      </c>
+      <c r="G12" s="107" t="s">
+        <v>205</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="I12" s="108">
+        <v>30500000</v>
+      </c>
+      <c r="J12" s="6">
+        <v>32</v>
+      </c>
+      <c r="K12" s="6">
+        <v>3</v>
+      </c>
+      <c r="L12">
+        <v>37.5</v>
+      </c>
+      <c r="M12" s="109">
+        <v>976000000</v>
+      </c>
       <c r="N12" s="6"/>
       <c r="O12" s="6"/>
       <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
+      <c r="Q12" s="109">
+        <v>457500000</v>
+      </c>
+      <c r="R12" s="109">
+        <v>122000000</v>
+      </c>
+      <c r="S12" s="109">
+        <v>343125000</v>
+      </c>
       <c r="T12" s="6"/>
       <c r="U12" s="6"/>
       <c r="V12" s="6"/>
-      <c r="W12" s="6"/>
+      <c r="W12" s="109">
+        <v>1898625000</v>
+      </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="23">
@@ -23791,9 +23807,11 @@
       <c r="W18" s="6"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
+      <c r="A19" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B19" s="14" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -24019,7 +24037,7 @@
         <v>39</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -24121,33 +24139,40 @@
       <c r="W30" s="12"/>
     </row>
     <row r="31" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="111" t="s">
-        <v>194</v>
-      </c>
-      <c r="C31" s="112"/>
-      <c r="D31" s="112"/>
-      <c r="E31" s="112"/>
-      <c r="F31" s="112"/>
-      <c r="G31" s="112"/>
-      <c r="H31" s="112"/>
-      <c r="I31" s="112"/>
-      <c r="J31" s="112"/>
-      <c r="K31" s="112"/>
-      <c r="L31" s="112"/>
-      <c r="M31" s="112"/>
-      <c r="N31" s="112"/>
-      <c r="O31" s="112"/>
-      <c r="P31" s="112"/>
-      <c r="Q31" s="112"/>
-      <c r="R31" s="112"/>
-      <c r="S31" s="112"/>
-      <c r="T31" s="112"/>
-      <c r="U31" s="112"/>
-      <c r="V31" s="112"/>
-      <c r="W31" s="112"/>
+      <c r="B31" s="116" t="s">
+        <v>181</v>
+      </c>
+      <c r="C31" s="117"/>
+      <c r="D31" s="117"/>
+      <c r="E31" s="117"/>
+      <c r="F31" s="117"/>
+      <c r="G31" s="117"/>
+      <c r="H31" s="117"/>
+      <c r="I31" s="117"/>
+      <c r="J31" s="117"/>
+      <c r="K31" s="117"/>
+      <c r="L31" s="117"/>
+      <c r="M31" s="117"/>
+      <c r="N31" s="117"/>
+      <c r="O31" s="117"/>
+      <c r="P31" s="117"/>
+      <c r="Q31" s="117"/>
+      <c r="R31" s="117"/>
+      <c r="S31" s="117"/>
+      <c r="T31" s="117"/>
+      <c r="U31" s="117"/>
+      <c r="V31" s="117"/>
+      <c r="W31" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="B31:W31"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="J6:J8"/>
     <mergeCell ref="C1:W1"/>
     <mergeCell ref="H6:H8"/>
     <mergeCell ref="I6:I8"/>
@@ -24164,13 +24189,6 @@
     <mergeCell ref="K6:K8"/>
     <mergeCell ref="C2:W2"/>
     <mergeCell ref="C3:W3"/>
-    <mergeCell ref="B31:W31"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="J6:J8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="55" orientation="landscape" r:id="rId1"/>
@@ -24193,77 +24211,77 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="110" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="107"/>
-      <c r="O1" s="107"/>
-      <c r="P1" s="107"/>
-      <c r="Q1" s="107"/>
-      <c r="R1" s="107"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="110"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="110"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="97" t="s">
-        <v>200</v>
-      </c>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="97"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="97"/>
-      <c r="L2" s="97"/>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
-      <c r="P2" s="97"/>
-      <c r="Q2" s="97"/>
-      <c r="R2" s="97"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="97"/>
-      <c r="U2" s="97"/>
-      <c r="V2" s="97"/>
-      <c r="W2" s="97"/>
+      <c r="C2" s="130" t="s">
+        <v>187</v>
+      </c>
+      <c r="D2" s="130"/>
+      <c r="E2" s="130"/>
+      <c r="F2" s="130"/>
+      <c r="G2" s="130"/>
+      <c r="H2" s="130"/>
+      <c r="I2" s="130"/>
+      <c r="J2" s="130"/>
+      <c r="K2" s="130"/>
+      <c r="L2" s="130"/>
+      <c r="M2" s="130"/>
+      <c r="N2" s="130"/>
+      <c r="O2" s="130"/>
+      <c r="P2" s="130"/>
+      <c r="Q2" s="130"/>
+      <c r="R2" s="130"/>
+      <c r="S2" s="130"/>
+      <c r="T2" s="130"/>
+      <c r="U2" s="130"/>
+      <c r="V2" s="130"/>
+      <c r="W2" s="130"/>
     </row>
     <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
-      <c r="P3" s="93"/>
-      <c r="Q3" s="93"/>
-      <c r="R3" s="93"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115"/>
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="115"/>
     </row>
     <row r="4" spans="1:23" s="15" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:23" x14ac:dyDescent="0.3">
@@ -24273,87 +24291,87 @@
       <c r="R5" s="18"/>
     </row>
     <row r="6" spans="1:23" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="91" t="s">
+      <c r="A6" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="91" t="s">
+      <c r="B6" s="111" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="91" t="s">
+      <c r="C6" s="111" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="91" t="s">
+      <c r="D6" s="111" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="91" t="s">
+      <c r="E6" s="111" t="s">
         <v>102</v>
       </c>
-      <c r="F6" s="91" t="s">
+      <c r="F6" s="111" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="91" t="s">
+      <c r="H6" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="I6" s="91" t="s">
+      <c r="I6" s="111" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="91" t="s">
+      <c r="J6" s="111" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="91" t="s">
+      <c r="K6" s="111" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="91" t="s">
+      <c r="L6" s="111" t="s">
         <v>86</v>
       </c>
-      <c r="M6" s="91"/>
-      <c r="N6" s="91"/>
-      <c r="O6" s="91"/>
-      <c r="P6" s="91"/>
-      <c r="Q6" s="91"/>
-      <c r="R6" s="91" t="s">
+      <c r="M6" s="111"/>
+      <c r="N6" s="111"/>
+      <c r="O6" s="111"/>
+      <c r="P6" s="111"/>
+      <c r="Q6" s="111"/>
+      <c r="R6" s="111" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:23" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="91"/>
-      <c r="B7" s="91"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="91"/>
-      <c r="K7" s="91"/>
-      <c r="L7" s="91" t="s">
+      <c r="A7" s="111"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="111"/>
+      <c r="E7" s="111"/>
+      <c r="F7" s="111"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="111"/>
+      <c r="I7" s="111"/>
+      <c r="J7" s="111"/>
+      <c r="K7" s="111"/>
+      <c r="L7" s="111" t="s">
         <v>9</v>
       </c>
-      <c r="M7" s="91"/>
-      <c r="N7" s="91"/>
-      <c r="O7" s="91" t="s">
+      <c r="M7" s="111"/>
+      <c r="N7" s="111"/>
+      <c r="O7" s="111" t="s">
         <v>12</v>
       </c>
-      <c r="P7" s="91"/>
-      <c r="Q7" s="91"/>
-      <c r="R7" s="91"/>
+      <c r="P7" s="111"/>
+      <c r="Q7" s="111"/>
+      <c r="R7" s="111"/>
     </row>
     <row r="8" spans="1:23" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="91"/>
-      <c r="B8" s="91"/>
-      <c r="C8" s="91"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
-      <c r="K8" s="91"/>
+      <c r="A8" s="111"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="111"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="111"/>
+      <c r="G8" s="111"/>
+      <c r="H8" s="111"/>
+      <c r="I8" s="111"/>
+      <c r="J8" s="111"/>
+      <c r="K8" s="111"/>
       <c r="L8" s="7" t="s">
         <v>43</v>
       </c>
@@ -24372,9 +24390,9 @@
       <c r="Q8" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="R8" s="91"/>
-    </row>
-    <row r="9" spans="1:23" s="10" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="R8" s="111"/>
+    </row>
+    <row r="9" spans="1:23" s="10" customFormat="1" ht="10.199999999999999" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>1</v>
       </c>
@@ -24396,44 +24414,46 @@
       <c r="G9" s="9">
         <v>7</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="27">
         <v>8</v>
       </c>
       <c r="I9" s="9">
         <v>9</v>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="27">
         <v>10</v>
       </c>
       <c r="K9" s="9">
         <v>11</v>
       </c>
-      <c r="L9" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="N9" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="O9" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="P9" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q9" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="R9" s="9" t="s">
-        <v>109</v>
+      <c r="L9" s="27">
+        <v>12</v>
+      </c>
+      <c r="M9" s="9">
+        <v>13</v>
+      </c>
+      <c r="N9" s="27">
+        <v>14</v>
+      </c>
+      <c r="O9" s="9">
+        <v>15</v>
+      </c>
+      <c r="P9" s="27">
+        <v>16</v>
+      </c>
+      <c r="Q9" s="9">
+        <v>17</v>
+      </c>
+      <c r="R9" s="27">
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:23" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
+      <c r="A10" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B10" s="14" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -24682,9 +24702,11 @@
       <c r="W18" s="6"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
+      <c r="A19" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B19" s="14" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -25002,33 +25024,38 @@
       <c r="R30" s="12"/>
     </row>
     <row r="31" spans="1:23" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="131" t="s">
-        <v>201</v>
-      </c>
-      <c r="C31" s="132"/>
-      <c r="D31" s="132"/>
-      <c r="E31" s="132"/>
-      <c r="F31" s="132"/>
-      <c r="G31" s="132"/>
-      <c r="H31" s="132"/>
-      <c r="I31" s="132"/>
-      <c r="J31" s="132"/>
-      <c r="K31" s="132"/>
-      <c r="L31" s="132"/>
-      <c r="M31" s="132"/>
-      <c r="N31" s="132"/>
-      <c r="O31" s="132"/>
-      <c r="P31" s="132"/>
-      <c r="Q31" s="132"/>
-      <c r="R31" s="132"/>
-      <c r="S31" s="132"/>
-      <c r="T31" s="132"/>
-      <c r="U31" s="132"/>
-      <c r="V31" s="132"/>
-      <c r="W31" s="132"/>
+      <c r="B31" s="134" t="s">
+        <v>188</v>
+      </c>
+      <c r="C31" s="135"/>
+      <c r="D31" s="135"/>
+      <c r="E31" s="135"/>
+      <c r="F31" s="135"/>
+      <c r="G31" s="135"/>
+      <c r="H31" s="135"/>
+      <c r="I31" s="135"/>
+      <c r="J31" s="135"/>
+      <c r="K31" s="135"/>
+      <c r="L31" s="135"/>
+      <c r="M31" s="135"/>
+      <c r="N31" s="135"/>
+      <c r="O31" s="135"/>
+      <c r="P31" s="135"/>
+      <c r="Q31" s="135"/>
+      <c r="R31" s="135"/>
+      <c r="S31" s="135"/>
+      <c r="T31" s="135"/>
+      <c r="U31" s="135"/>
+      <c r="V31" s="135"/>
+      <c r="W31" s="135"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
     <mergeCell ref="B31:W31"/>
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="K6:K8"/>
@@ -25043,11 +25070,6 @@
     <mergeCell ref="H6:H8"/>
     <mergeCell ref="I6:I8"/>
     <mergeCell ref="C2:W2"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="70" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -25070,42 +25092,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="110" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="107"/>
-      <c r="O1" s="107"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
     </row>
     <row r="2" spans="1:23" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="122" t="s">
-        <v>202</v>
-      </c>
-      <c r="D2" s="122"/>
-      <c r="E2" s="122"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="122"/>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="122"/>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
+      <c r="C2" s="142" t="s">
+        <v>189</v>
+      </c>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -25117,21 +25139,21 @@
         <v>7</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115"/>
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
       <c r="P3" s="19"/>
       <c r="Q3" s="19"/>
       <c r="R3" s="19"/>
@@ -25164,77 +25186,77 @@
       <c r="N5" s="21"/>
     </row>
     <row r="6" spans="1:23" s="1" customFormat="1" ht="32.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="91" t="s">
+      <c r="A6" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="91" t="s">
+      <c r="B6" s="111" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="91" t="s">
+      <c r="C6" s="111" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="91" t="s">
+      <c r="D6" s="111" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="91" t="s">
+      <c r="E6" s="111" t="s">
         <v>102</v>
       </c>
-      <c r="F6" s="91" t="s">
+      <c r="F6" s="111" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="91" t="s">
+      <c r="H6" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="91" t="s">
+      <c r="I6" s="111" t="s">
         <v>49</v>
       </c>
-      <c r="J6" s="91" t="s">
-        <v>118</v>
-      </c>
-      <c r="K6" s="91" t="s">
-        <v>119</v>
-      </c>
-      <c r="L6" s="116" t="s">
+      <c r="J6" s="111" t="s">
+        <v>111</v>
+      </c>
+      <c r="K6" s="111" t="s">
+        <v>112</v>
+      </c>
+      <c r="L6" s="136" t="s">
         <v>48</v>
       </c>
-      <c r="M6" s="117"/>
-      <c r="N6" s="118"/>
-      <c r="O6" s="91" t="s">
+      <c r="M6" s="137"/>
+      <c r="N6" s="138"/>
+      <c r="O6" s="111" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:23" s="1" customFormat="1" ht="31.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="91"/>
-      <c r="B7" s="91"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="91"/>
-      <c r="K7" s="91"/>
-      <c r="L7" s="119"/>
-      <c r="M7" s="120"/>
-      <c r="N7" s="121"/>
-      <c r="O7" s="91"/>
+      <c r="A7" s="111"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="111"/>
+      <c r="E7" s="111"/>
+      <c r="F7" s="111"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="111"/>
+      <c r="I7" s="111"/>
+      <c r="J7" s="111"/>
+      <c r="K7" s="111"/>
+      <c r="L7" s="139"/>
+      <c r="M7" s="140"/>
+      <c r="N7" s="141"/>
+      <c r="O7" s="111"/>
     </row>
     <row r="8" spans="1:23" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="91"/>
-      <c r="B8" s="91"/>
-      <c r="C8" s="91"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
-      <c r="K8" s="91"/>
+      <c r="A8" s="111"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="111"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="111"/>
+      <c r="G8" s="111"/>
+      <c r="H8" s="111"/>
+      <c r="I8" s="111"/>
+      <c r="J8" s="111"/>
+      <c r="K8" s="111"/>
       <c r="L8" s="5" t="s">
         <v>20</v>
       </c>
@@ -25244,9 +25266,9 @@
       <c r="N8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="O8" s="91"/>
-    </row>
-    <row r="9" spans="1:23" s="10" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="O8" s="111"/>
+    </row>
+    <row r="9" spans="1:23" s="10" customFormat="1" ht="10.199999999999999" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>1</v>
       </c>
@@ -25260,7 +25282,7 @@
         <v>4</v>
       </c>
       <c r="E9" s="9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" s="9">
         <v>6</v>
@@ -25274,29 +25296,31 @@
       <c r="I9" s="9">
         <v>9</v>
       </c>
-      <c r="J9" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="L9" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="N9" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="O9" s="9" t="s">
-        <v>122</v>
+      <c r="J9" s="9">
+        <v>10</v>
+      </c>
+      <c r="K9" s="9">
+        <v>11</v>
+      </c>
+      <c r="L9" s="9">
+        <v>12</v>
+      </c>
+      <c r="M9" s="9">
+        <v>13</v>
+      </c>
+      <c r="N9" s="9">
+        <v>14</v>
+      </c>
+      <c r="O9" s="9">
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:23" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
+      <c r="A10" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B10" s="14" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -25545,9 +25569,11 @@
       <c r="W18" s="6"/>
     </row>
     <row r="19" spans="1:23" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
+      <c r="A19" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B19" s="14" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
@@ -25811,14 +25837,6 @@
       <c r="M28" s="11"/>
       <c r="N28" s="11"/>
       <c r="O28" s="11"/>
-      <c r="P28" s="133"/>
-      <c r="Q28" s="133"/>
-      <c r="R28" s="133"/>
-      <c r="S28" s="133"/>
-      <c r="T28" s="133"/>
-      <c r="U28" s="133"/>
-      <c r="V28" s="133"/>
-      <c r="W28" s="133"/>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" s="23" t="s">
@@ -25859,33 +25877,38 @@
       <c r="O30" s="12"/>
     </row>
     <row r="31" spans="1:23" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="131" t="s">
-        <v>201</v>
-      </c>
-      <c r="C31" s="132"/>
-      <c r="D31" s="132"/>
-      <c r="E31" s="132"/>
-      <c r="F31" s="132"/>
-      <c r="G31" s="132"/>
-      <c r="H31" s="132"/>
-      <c r="I31" s="132"/>
-      <c r="J31" s="132"/>
-      <c r="K31" s="132"/>
-      <c r="L31" s="132"/>
-      <c r="M31" s="132"/>
-      <c r="N31" s="132"/>
-      <c r="O31" s="132"/>
-      <c r="P31" s="132"/>
-      <c r="Q31" s="132"/>
-      <c r="R31" s="132"/>
-      <c r="S31" s="132"/>
-      <c r="T31" s="132"/>
-      <c r="U31" s="132"/>
-      <c r="V31" s="132"/>
-      <c r="W31" s="132"/>
+      <c r="B31" s="134" t="s">
+        <v>188</v>
+      </c>
+      <c r="C31" s="135"/>
+      <c r="D31" s="135"/>
+      <c r="E31" s="135"/>
+      <c r="F31" s="135"/>
+      <c r="G31" s="135"/>
+      <c r="H31" s="135"/>
+      <c r="I31" s="135"/>
+      <c r="J31" s="135"/>
+      <c r="K31" s="135"/>
+      <c r="L31" s="135"/>
+      <c r="M31" s="135"/>
+      <c r="N31" s="135"/>
+      <c r="O31" s="135"/>
+      <c r="P31" s="135"/>
+      <c r="Q31" s="135"/>
+      <c r="R31" s="135"/>
+      <c r="S31" s="135"/>
+      <c r="T31" s="135"/>
+      <c r="U31" s="135"/>
+      <c r="V31" s="135"/>
+      <c r="W31" s="135"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
     <mergeCell ref="B31:W31"/>
     <mergeCell ref="L6:N7"/>
     <mergeCell ref="C1:O1"/>
@@ -25898,11 +25921,6 @@
     <mergeCell ref="J6:J8"/>
     <mergeCell ref="K6:K8"/>
     <mergeCell ref="F6:F8"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="65" orientation="landscape" r:id="rId1"/>
@@ -25923,66 +25941,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C1" s="107" t="s">
-        <v>203</v>
-      </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="107"/>
-      <c r="O1" s="107"/>
-      <c r="P1" s="107"/>
+      <c r="C1" s="110" t="s">
+        <v>190</v>
+      </c>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="110"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="107" t="s">
-        <v>204</v>
-      </c>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
-      <c r="M2" s="107"/>
-      <c r="N2" s="107"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="107"/>
+      <c r="C2" s="110" t="s">
+        <v>191</v>
+      </c>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
+      <c r="L2" s="110"/>
+      <c r="M2" s="110"/>
+      <c r="N2" s="110"/>
+      <c r="O2" s="110"/>
+      <c r="P2" s="110"/>
     </row>
     <row r="3" spans="1:16" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
-      <c r="P3" s="93"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115"/>
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
     </row>
     <row r="4" spans="1:16" s="15" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="C4" s="16"/>
@@ -25993,68 +26011,68 @@
       <c r="O4" s="16"/>
     </row>
     <row r="5" spans="1:16" s="1" customFormat="1" ht="24.45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="91" t="s">
+      <c r="A5" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="91" t="s">
+      <c r="B5" s="111" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="91" t="s">
+      <c r="C5" s="111" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="91" t="s">
+      <c r="D5" s="111" t="s">
         <v>95</v>
       </c>
-      <c r="E5" s="113" t="s">
+      <c r="E5" s="112" t="s">
         <v>94</v>
       </c>
-      <c r="F5" s="114"/>
-      <c r="G5" s="114"/>
-      <c r="H5" s="115"/>
-      <c r="I5" s="116" t="s">
+      <c r="F5" s="113"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="114"/>
+      <c r="I5" s="136" t="s">
         <v>99</v>
       </c>
-      <c r="J5" s="118"/>
-      <c r="K5" s="116" t="s">
-        <v>128</v>
-      </c>
-      <c r="L5" s="117"/>
-      <c r="M5" s="117"/>
-      <c r="N5" s="118"/>
-      <c r="O5" s="123" t="s">
+      <c r="J5" s="138"/>
+      <c r="K5" s="136" t="s">
+        <v>115</v>
+      </c>
+      <c r="L5" s="137"/>
+      <c r="M5" s="137"/>
+      <c r="N5" s="138"/>
+      <c r="O5" s="143" t="s">
         <v>90</v>
       </c>
-      <c r="P5" s="123" t="s">
-        <v>132</v>
+      <c r="P5" s="143" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="91"/>
-      <c r="B6" s="91"/>
-      <c r="C6" s="91"/>
-      <c r="D6" s="91"/>
-      <c r="E6" s="113" t="s">
+      <c r="A6" s="111"/>
+      <c r="B6" s="111"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="111"/>
+      <c r="E6" s="112" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="115"/>
-      <c r="G6" s="113" t="s">
+      <c r="F6" s="114"/>
+      <c r="G6" s="112" t="s">
         <v>101</v>
       </c>
-      <c r="H6" s="115"/>
-      <c r="I6" s="119"/>
-      <c r="J6" s="121"/>
-      <c r="K6" s="126"/>
-      <c r="L6" s="127"/>
-      <c r="M6" s="127"/>
-      <c r="N6" s="128"/>
-      <c r="O6" s="124"/>
-      <c r="P6" s="124"/>
+      <c r="H6" s="114"/>
+      <c r="I6" s="139"/>
+      <c r="J6" s="141"/>
+      <c r="K6" s="146"/>
+      <c r="L6" s="147"/>
+      <c r="M6" s="147"/>
+      <c r="N6" s="148"/>
+      <c r="O6" s="144"/>
+      <c r="P6" s="144"/>
     </row>
     <row r="7" spans="1:16" ht="89.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="91"/>
-      <c r="B7" s="91"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
+      <c r="A7" s="111"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="111"/>
       <c r="E7" s="5" t="s">
         <v>98</v>
       </c>
@@ -26068,25 +26086,25 @@
         <v>96</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="O7" s="125"/>
-      <c r="P7" s="125"/>
+        <v>120</v>
+      </c>
+      <c r="O7" s="145"/>
+      <c r="P7" s="145"/>
     </row>
     <row r="8" spans="1:16" s="10" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
@@ -26141,7 +26159,7 @@
     <row r="9" spans="1:16" s="2" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A9" s="14"/>
       <c r="B9" s="14" t="s">
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -26159,9 +26177,11 @@
       <c r="P9" s="14"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
+      <c r="A10" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B10" s="14" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -26347,9 +26367,11 @@
       <c r="P18" s="6"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
+      <c r="A19" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B19" s="14" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -26535,7 +26557,7 @@
     <row r="28" spans="1:16" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A28" s="23"/>
       <c r="B28" s="14" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
@@ -26553,9 +26575,11 @@
       <c r="P28" s="6"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A29" s="14"/>
+      <c r="A29" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B29" s="14" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -26741,9 +26765,11 @@
       <c r="P37" s="6"/>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A38" s="14"/>
+      <c r="A38" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="B38" s="14" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
@@ -26929,7 +26955,7 @@
       <c r="P46" s="6"/>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A47" s="134"/>
+      <c r="A47" s="91"/>
       <c r="B47" s="11"/>
       <c r="C47" s="11"/>
       <c r="D47" s="11"/>
@@ -26985,26 +27011,31 @@
       <c r="P49" s="12"/>
     </row>
     <row r="50" spans="1:16" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="111" t="s">
-        <v>207</v>
-      </c>
-      <c r="C50" s="112"/>
-      <c r="D50" s="112"/>
-      <c r="E50" s="112"/>
-      <c r="F50" s="112"/>
-      <c r="G50" s="112"/>
-      <c r="H50" s="112"/>
-      <c r="I50" s="112"/>
-      <c r="J50" s="112"/>
-      <c r="K50" s="112"/>
-      <c r="L50" s="112"/>
-      <c r="M50" s="112"/>
-      <c r="N50" s="112"/>
-      <c r="O50" s="112"/>
-      <c r="P50" s="112"/>
+      <c r="B50" s="116" t="s">
+        <v>194</v>
+      </c>
+      <c r="C50" s="117"/>
+      <c r="D50" s="117"/>
+      <c r="E50" s="117"/>
+      <c r="F50" s="117"/>
+      <c r="G50" s="117"/>
+      <c r="H50" s="117"/>
+      <c r="I50" s="117"/>
+      <c r="J50" s="117"/>
+      <c r="K50" s="117"/>
+      <c r="L50" s="117"/>
+      <c r="M50" s="117"/>
+      <c r="N50" s="117"/>
+      <c r="O50" s="117"/>
+      <c r="P50" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B50:P50"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I5:J6"/>
     <mergeCell ref="C1:P1"/>
     <mergeCell ref="C2:P2"/>
     <mergeCell ref="C3:P3"/>
@@ -27015,11 +27046,6 @@
     <mergeCell ref="O5:O7"/>
     <mergeCell ref="P5:P7"/>
     <mergeCell ref="K5:N6"/>
-    <mergeCell ref="B50:P50"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I5:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="55" orientation="landscape" r:id="rId1"/>
@@ -27036,9 +27062,9 @@
   <cols>
     <col min="1" max="1" width="5.09765625" customWidth="1"/>
     <col min="2" max="2" width="25" style="12" customWidth="1"/>
-    <col min="3" max="3" width="10.69921875" style="149" customWidth="1"/>
-    <col min="4" max="4" width="10.69921875" style="133" customWidth="1"/>
-    <col min="5" max="5" width="10.09765625" style="133" customWidth="1"/>
+    <col min="3" max="3" width="10.69921875" style="101" customWidth="1"/>
+    <col min="4" max="4" width="10.69921875" customWidth="1"/>
+    <col min="5" max="5" width="10.09765625" customWidth="1"/>
     <col min="6" max="6" width="12.19921875" customWidth="1"/>
     <col min="7" max="7" width="11.59765625" customWidth="1"/>
     <col min="8" max="8" width="8.296875" customWidth="1"/>
@@ -27053,127 +27079,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="154" t="s">
-        <v>180</v>
-      </c>
-      <c r="B1" s="154"/>
-      <c r="C1" s="154"/>
-      <c r="D1" s="154"/>
-      <c r="E1" s="154"/>
-      <c r="F1" s="154"/>
-      <c r="G1" s="154"/>
-      <c r="H1" s="154"/>
-      <c r="I1" s="154"/>
-      <c r="J1" s="154"/>
-      <c r="K1" s="154"/>
-      <c r="L1" s="154"/>
-      <c r="M1" s="154"/>
-      <c r="N1" s="154"/>
-      <c r="O1" s="154"/>
-      <c r="P1" s="154"/>
-      <c r="Q1" s="154"/>
-      <c r="R1" s="154"/>
-      <c r="S1" s="154"/>
-      <c r="T1" s="154"/>
-      <c r="U1" s="154"/>
-      <c r="V1" s="154"/>
-    </row>
-    <row r="2" spans="1:24" s="157" customFormat="1" x14ac:dyDescent="0.3"/>
+      <c r="A1" s="149" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" s="149"/>
+      <c r="C1" s="149"/>
+      <c r="D1" s="149"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="149"/>
+      <c r="J1" s="149"/>
+      <c r="K1" s="149"/>
+      <c r="L1" s="149"/>
+      <c r="M1" s="149"/>
+      <c r="N1" s="149"/>
+      <c r="O1" s="149"/>
+      <c r="P1" s="149"/>
+      <c r="Q1" s="149"/>
+      <c r="R1" s="149"/>
+      <c r="S1" s="149"/>
+      <c r="T1" s="149"/>
+      <c r="U1" s="149"/>
+      <c r="V1" s="149"/>
+    </row>
+    <row r="2" spans="1:24" s="106" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="126" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="140" t="s">
+      <c r="A3" s="146" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="151" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="121" t="s">
-        <v>212</v>
-      </c>
-      <c r="D3" s="124" t="s">
-        <v>214</v>
-      </c>
-      <c r="E3" s="123" t="s">
-        <v>142</v>
-      </c>
-      <c r="F3" s="136" t="s">
-        <v>213</v>
-      </c>
-      <c r="G3" s="138"/>
-      <c r="H3" s="137"/>
-      <c r="I3" s="139" t="s">
-        <v>140</v>
-      </c>
-      <c r="J3" s="139"/>
-      <c r="K3" s="124" t="s">
-        <v>208</v>
-      </c>
-      <c r="L3" s="124" t="s">
-        <v>209</v>
-      </c>
-      <c r="M3" s="125" t="s">
-        <v>139</v>
-      </c>
-      <c r="N3" s="125"/>
-      <c r="O3" s="125"/>
-      <c r="P3" s="125"/>
-      <c r="Q3" s="125"/>
-      <c r="R3" s="125"/>
-      <c r="S3" s="125"/>
-      <c r="T3" s="125"/>
-      <c r="U3" s="125"/>
-      <c r="V3" s="125"/>
+      <c r="C3" s="141" t="s">
+        <v>199</v>
+      </c>
+      <c r="D3" s="144" t="s">
+        <v>201</v>
+      </c>
+      <c r="E3" s="143" t="s">
+        <v>129</v>
+      </c>
+      <c r="F3" s="153" t="s">
+        <v>200</v>
+      </c>
+      <c r="G3" s="154"/>
+      <c r="H3" s="155"/>
+      <c r="I3" s="150" t="s">
+        <v>127</v>
+      </c>
+      <c r="J3" s="150"/>
+      <c r="K3" s="144" t="s">
+        <v>195</v>
+      </c>
+      <c r="L3" s="144" t="s">
+        <v>196</v>
+      </c>
+      <c r="M3" s="145" t="s">
+        <v>126</v>
+      </c>
+      <c r="N3" s="145"/>
+      <c r="O3" s="145"/>
+      <c r="P3" s="145"/>
+      <c r="Q3" s="145"/>
+      <c r="R3" s="145"/>
+      <c r="S3" s="145"/>
+      <c r="T3" s="145"/>
+      <c r="U3" s="145"/>
+      <c r="V3" s="145"/>
       <c r="W3" s="30"/>
       <c r="X3" s="30"/>
     </row>
-    <row r="4" spans="1:24" s="135" customFormat="1" ht="162" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="119"/>
-      <c r="B4" s="92"/>
-      <c r="C4" s="115"/>
-      <c r="D4" s="125"/>
-      <c r="E4" s="125"/>
+    <row r="4" spans="1:24" s="92" customFormat="1" ht="162" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="139"/>
+      <c r="B4" s="152"/>
+      <c r="C4" s="114"/>
+      <c r="D4" s="145"/>
+      <c r="E4" s="145"/>
       <c r="F4" s="5" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>97</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="K4" s="125"/>
-      <c r="L4" s="125"/>
+        <v>131</v>
+      </c>
+      <c r="K4" s="145"/>
+      <c r="L4" s="145"/>
       <c r="M4" s="5" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>210</v>
+        <v>197</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="V4" s="5" t="s">
         <v>36</v>
@@ -27182,67 +27208,67 @@
       <c r="X4" s="73"/>
     </row>
     <row r="5" spans="1:24" s="90" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A5" s="144">
+      <c r="A5" s="96">
         <v>1</v>
       </c>
       <c r="B5" s="89">
         <v>2</v>
       </c>
-      <c r="C5" s="144">
+      <c r="C5" s="96">
         <v>3</v>
       </c>
       <c r="D5" s="89">
         <v>4</v>
       </c>
-      <c r="E5" s="144">
+      <c r="E5" s="96">
         <v>5</v>
       </c>
       <c r="F5" s="89">
         <v>6</v>
       </c>
-      <c r="G5" s="144">
+      <c r="G5" s="96">
         <v>7</v>
       </c>
       <c r="H5" s="89">
         <v>8</v>
       </c>
-      <c r="I5" s="144">
+      <c r="I5" s="96">
         <v>9</v>
       </c>
       <c r="J5" s="89">
         <v>10</v>
       </c>
-      <c r="K5" s="144">
+      <c r="K5" s="96">
         <v>11</v>
       </c>
       <c r="L5" s="89">
         <v>12</v>
       </c>
-      <c r="M5" s="144">
+      <c r="M5" s="96">
         <v>13</v>
       </c>
       <c r="N5" s="89">
         <v>14</v>
       </c>
-      <c r="O5" s="144">
+      <c r="O5" s="96">
         <v>15</v>
       </c>
       <c r="P5" s="89">
         <v>16</v>
       </c>
-      <c r="Q5" s="144">
+      <c r="Q5" s="96">
         <v>17</v>
       </c>
       <c r="R5" s="89">
         <v>18</v>
       </c>
-      <c r="S5" s="144">
+      <c r="S5" s="96">
         <v>19</v>
       </c>
       <c r="T5" s="89">
         <v>20</v>
       </c>
-      <c r="U5" s="144">
+      <c r="U5" s="96">
         <v>21</v>
       </c>
       <c r="V5" s="89">
@@ -27252,7 +27278,7 @@
     <row r="6" spans="1:24" s="90" customFormat="1" ht="31.2" x14ac:dyDescent="0.25">
       <c r="A6" s="78"/>
       <c r="B6" s="5" t="s">
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="C6" s="77"/>
       <c r="D6" s="77"/>
@@ -27276,9 +27302,11 @@
       <c r="V6" s="89"/>
     </row>
     <row r="7" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="78"/>
+      <c r="A7" s="78" t="s">
+        <v>208</v>
+      </c>
       <c r="B7" s="5" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C7" s="77"/>
       <c r="D7" s="77"/>
@@ -27302,15 +27330,15 @@
       <c r="V7" s="89"/>
     </row>
     <row r="8" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="145" t="s">
+      <c r="A8" s="97" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="141" t="s">
+      <c r="B8" s="93" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="148"/>
-      <c r="D8" s="148"/>
-      <c r="E8" s="148"/>
+      <c r="C8" s="100"/>
+      <c r="D8" s="100"/>
+      <c r="E8" s="100"/>
       <c r="F8" s="89"/>
       <c r="G8" s="88"/>
       <c r="H8" s="88"/>
@@ -27330,15 +27358,15 @@
       <c r="V8" s="89"/>
     </row>
     <row r="9" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="146">
+      <c r="A9" s="98">
         <v>1</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="149"/>
-      <c r="D9" s="149"/>
-      <c r="E9" s="149"/>
+      <c r="C9" s="101"/>
+      <c r="D9" s="101"/>
+      <c r="E9" s="101"/>
       <c r="F9" s="89"/>
       <c r="G9" s="88"/>
       <c r="H9" s="88"/>
@@ -27358,13 +27386,13 @@
       <c r="V9" s="89"/>
     </row>
     <row r="10" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="146">
+      <c r="A10" s="98">
         <v>2</v>
       </c>
       <c r="B10" s="12"/>
-      <c r="C10" s="149"/>
-      <c r="D10" s="149"/>
-      <c r="E10" s="149"/>
+      <c r="C10" s="101"/>
+      <c r="D10" s="101"/>
+      <c r="E10" s="101"/>
       <c r="F10" s="89"/>
       <c r="G10" s="88"/>
       <c r="H10" s="88"/>
@@ -27384,13 +27412,13 @@
       <c r="V10" s="89"/>
     </row>
     <row r="11" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="146" t="s">
+      <c r="A11" s="98" t="s">
         <v>39</v>
       </c>
       <c r="B11" s="12"/>
-      <c r="C11" s="149"/>
-      <c r="D11" s="149"/>
-      <c r="E11" s="149"/>
+      <c r="C11" s="101"/>
+      <c r="D11" s="101"/>
+      <c r="E11" s="101"/>
       <c r="F11" s="89"/>
       <c r="G11" s="88"/>
       <c r="H11" s="88"/>
@@ -27410,15 +27438,15 @@
       <c r="V11" s="89"/>
     </row>
     <row r="12" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="145" t="s">
+      <c r="A12" s="97" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="141" t="s">
+      <c r="B12" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="148"/>
-      <c r="D12" s="148"/>
-      <c r="E12" s="148"/>
+      <c r="C12" s="100"/>
+      <c r="D12" s="100"/>
+      <c r="E12" s="100"/>
       <c r="F12" s="89"/>
       <c r="G12" s="88"/>
       <c r="H12" s="88"/>
@@ -27438,15 +27466,15 @@
       <c r="V12" s="89"/>
     </row>
     <row r="13" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="146">
+      <c r="A13" s="98">
         <v>1</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="149"/>
-      <c r="D13" s="149"/>
-      <c r="E13" s="149"/>
+      <c r="C13" s="101"/>
+      <c r="D13" s="101"/>
+      <c r="E13" s="101"/>
       <c r="F13" s="89"/>
       <c r="G13" s="88"/>
       <c r="H13" s="88"/>
@@ -27466,13 +27494,13 @@
       <c r="V13" s="89"/>
     </row>
     <row r="14" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="146">
+      <c r="A14" s="98">
         <v>2</v>
       </c>
       <c r="B14" s="12"/>
-      <c r="C14" s="149"/>
-      <c r="D14" s="149"/>
-      <c r="E14" s="149"/>
+      <c r="C14" s="101"/>
+      <c r="D14" s="101"/>
+      <c r="E14" s="101"/>
       <c r="F14" s="89"/>
       <c r="G14" s="88"/>
       <c r="H14" s="88"/>
@@ -27492,13 +27520,13 @@
       <c r="V14" s="89"/>
     </row>
     <row r="15" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="146" t="s">
+      <c r="A15" s="98" t="s">
         <v>39</v>
       </c>
       <c r="B15" s="12"/>
-      <c r="C15" s="149"/>
-      <c r="D15" s="149"/>
-      <c r="E15" s="149"/>
+      <c r="C15" s="101"/>
+      <c r="D15" s="101"/>
+      <c r="E15" s="101"/>
       <c r="F15" s="89"/>
       <c r="G15" s="88"/>
       <c r="H15" s="88"/>
@@ -27518,9 +27546,11 @@
       <c r="V15" s="89"/>
     </row>
     <row r="16" spans="1:24" s="90" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="78"/>
+      <c r="A16" s="78" t="s">
+        <v>208</v>
+      </c>
       <c r="B16" s="5" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="C16" s="77"/>
       <c r="D16" s="77"/>
@@ -27544,15 +27574,15 @@
       <c r="V16" s="89"/>
     </row>
     <row r="17" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="145" t="s">
+      <c r="A17" s="97" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="141" t="s">
+      <c r="B17" s="93" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="148"/>
-      <c r="D17" s="148"/>
-      <c r="E17" s="148"/>
+      <c r="C17" s="100"/>
+      <c r="D17" s="100"/>
+      <c r="E17" s="100"/>
       <c r="F17" s="89"/>
       <c r="G17" s="88"/>
       <c r="H17" s="88"/>
@@ -27572,15 +27602,15 @@
       <c r="V17" s="89"/>
     </row>
     <row r="18" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="146">
+      <c r="A18" s="98">
         <v>1</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="149"/>
-      <c r="D18" s="149"/>
-      <c r="E18" s="149"/>
+      <c r="C18" s="101"/>
+      <c r="D18" s="101"/>
+      <c r="E18" s="101"/>
       <c r="F18" s="89"/>
       <c r="G18" s="88"/>
       <c r="H18" s="88"/>
@@ -27600,13 +27630,13 @@
       <c r="V18" s="89"/>
     </row>
     <row r="19" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="146">
+      <c r="A19" s="98">
         <v>2</v>
       </c>
       <c r="B19" s="12"/>
-      <c r="C19" s="149"/>
-      <c r="D19" s="149"/>
-      <c r="E19" s="149"/>
+      <c r="C19" s="101"/>
+      <c r="D19" s="101"/>
+      <c r="E19" s="101"/>
       <c r="F19" s="89"/>
       <c r="G19" s="88"/>
       <c r="H19" s="88"/>
@@ -27626,13 +27656,13 @@
       <c r="V19" s="89"/>
     </row>
     <row r="20" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="146" t="s">
+      <c r="A20" s="98" t="s">
         <v>39</v>
       </c>
       <c r="B20" s="12"/>
-      <c r="C20" s="149"/>
-      <c r="D20" s="149"/>
-      <c r="E20" s="149"/>
+      <c r="C20" s="101"/>
+      <c r="D20" s="101"/>
+      <c r="E20" s="101"/>
       <c r="F20" s="89"/>
       <c r="G20" s="88"/>
       <c r="H20" s="88"/>
@@ -27652,15 +27682,15 @@
       <c r="V20" s="89"/>
     </row>
     <row r="21" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="145" t="s">
+      <c r="A21" s="97" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="141" t="s">
+      <c r="B21" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="148"/>
-      <c r="D21" s="148"/>
-      <c r="E21" s="148"/>
+      <c r="C21" s="100"/>
+      <c r="D21" s="100"/>
+      <c r="E21" s="100"/>
       <c r="F21" s="89"/>
       <c r="G21" s="88"/>
       <c r="H21" s="88"/>
@@ -27680,15 +27710,15 @@
       <c r="V21" s="89"/>
     </row>
     <row r="22" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="146">
+      <c r="A22" s="98">
         <v>1</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="149"/>
-      <c r="D22" s="149"/>
-      <c r="E22" s="149"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="101"/>
+      <c r="E22" s="101"/>
       <c r="F22" s="89"/>
       <c r="G22" s="88"/>
       <c r="H22" s="88"/>
@@ -27708,13 +27738,13 @@
       <c r="V22" s="89"/>
     </row>
     <row r="23" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="146">
+      <c r="A23" s="98">
         <v>2</v>
       </c>
       <c r="B23" s="12"/>
-      <c r="C23" s="149"/>
-      <c r="D23" s="149"/>
-      <c r="E23" s="149"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="101"/>
+      <c r="E23" s="101"/>
       <c r="F23" s="89"/>
       <c r="G23" s="88"/>
       <c r="H23" s="88"/>
@@ -27734,11 +27764,11 @@
       <c r="V23" s="89"/>
     </row>
     <row r="24" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="146"/>
+      <c r="A24" s="98"/>
       <c r="B24" s="12"/>
-      <c r="C24" s="149"/>
-      <c r="D24" s="149"/>
-      <c r="E24" s="149"/>
+      <c r="C24" s="101"/>
+      <c r="D24" s="101"/>
+      <c r="E24" s="101"/>
       <c r="F24" s="89"/>
       <c r="G24" s="88"/>
       <c r="H24" s="88"/>
@@ -27758,9 +27788,9 @@
       <c r="V24" s="89"/>
     </row>
     <row r="25" spans="1:22" s="90" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="146"/>
+      <c r="A25" s="98"/>
       <c r="B25" s="5" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="C25" s="77"/>
       <c r="D25" s="77"/>
@@ -27784,9 +27814,11 @@
       <c r="V25" s="89"/>
     </row>
     <row r="26" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="78"/>
+      <c r="A26" s="78" t="s">
+        <v>208</v>
+      </c>
       <c r="B26" s="5" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C26" s="77"/>
       <c r="D26" s="77"/>
@@ -27810,15 +27842,15 @@
       <c r="V26" s="89"/>
     </row>
     <row r="27" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="145" t="s">
+      <c r="A27" s="97" t="s">
         <v>37</v>
       </c>
-      <c r="B27" s="141" t="s">
+      <c r="B27" s="93" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="148"/>
-      <c r="D27" s="148"/>
-      <c r="E27" s="148"/>
+      <c r="C27" s="100"/>
+      <c r="D27" s="100"/>
+      <c r="E27" s="100"/>
       <c r="F27" s="89"/>
       <c r="G27" s="88"/>
       <c r="H27" s="88"/>
@@ -27838,15 +27870,15 @@
       <c r="V27" s="89"/>
     </row>
     <row r="28" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="146">
+      <c r="A28" s="98">
         <v>1</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="149"/>
-      <c r="D28" s="149"/>
-      <c r="E28" s="149"/>
+      <c r="C28" s="101"/>
+      <c r="D28" s="101"/>
+      <c r="E28" s="101"/>
       <c r="F28" s="89"/>
       <c r="G28" s="88"/>
       <c r="H28" s="88"/>
@@ -27866,13 +27898,13 @@
       <c r="V28" s="89"/>
     </row>
     <row r="29" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="146">
+      <c r="A29" s="98">
         <v>2</v>
       </c>
       <c r="B29" s="12"/>
-      <c r="C29" s="149"/>
-      <c r="D29" s="149"/>
-      <c r="E29" s="149"/>
+      <c r="C29" s="101"/>
+      <c r="D29" s="101"/>
+      <c r="E29" s="101"/>
       <c r="F29" s="89"/>
       <c r="G29" s="88"/>
       <c r="H29" s="88"/>
@@ -27892,13 +27924,13 @@
       <c r="V29" s="89"/>
     </row>
     <row r="30" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="146" t="s">
+      <c r="A30" s="98" t="s">
         <v>39</v>
       </c>
       <c r="B30" s="12"/>
-      <c r="C30" s="149"/>
-      <c r="D30" s="149"/>
-      <c r="E30" s="149"/>
+      <c r="C30" s="101"/>
+      <c r="D30" s="101"/>
+      <c r="E30" s="101"/>
       <c r="F30" s="89"/>
       <c r="G30" s="88"/>
       <c r="H30" s="88"/>
@@ -27918,15 +27950,15 @@
       <c r="V30" s="89"/>
     </row>
     <row r="31" spans="1:22" s="90" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="145" t="s">
+      <c r="A31" s="97" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="141" t="s">
+      <c r="B31" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="148"/>
-      <c r="D31" s="148"/>
-      <c r="E31" s="148"/>
+      <c r="C31" s="100"/>
+      <c r="D31" s="100"/>
+      <c r="E31" s="100"/>
       <c r="F31" s="89"/>
       <c r="G31" s="88"/>
       <c r="H31" s="88"/>
@@ -27946,15 +27978,15 @@
       <c r="V31" s="89"/>
     </row>
     <row r="32" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="146">
+      <c r="A32" s="98">
         <v>1</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C32" s="149"/>
-      <c r="D32" s="149"/>
-      <c r="E32" s="149"/>
+      <c r="C32" s="101"/>
+      <c r="D32" s="101"/>
+      <c r="E32" s="101"/>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
       <c r="H32" s="5"/>
@@ -27974,13 +28006,13 @@
       <c r="V32" s="5"/>
     </row>
     <row r="33" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="146">
+      <c r="A33" s="98">
         <v>2</v>
       </c>
       <c r="B33" s="12"/>
-      <c r="C33" s="149"/>
-      <c r="D33" s="149"/>
-      <c r="E33" s="149"/>
+      <c r="C33" s="101"/>
+      <c r="D33" s="101"/>
+      <c r="E33" s="101"/>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
@@ -28000,13 +28032,13 @@
       <c r="V33" s="5"/>
     </row>
     <row r="34" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="146" t="s">
+      <c r="A34" s="98" t="s">
         <v>39</v>
       </c>
       <c r="B34" s="12"/>
-      <c r="C34" s="149"/>
-      <c r="D34" s="149"/>
-      <c r="E34" s="149"/>
+      <c r="C34" s="101"/>
+      <c r="D34" s="101"/>
+      <c r="E34" s="101"/>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
       <c r="H34" s="5"/>
@@ -28026,9 +28058,11 @@
       <c r="V34" s="5"/>
     </row>
     <row r="35" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="78"/>
+      <c r="A35" s="78" t="s">
+        <v>208</v>
+      </c>
       <c r="B35" s="5" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="C35" s="77"/>
       <c r="D35" s="77"/>
@@ -28052,15 +28086,15 @@
       <c r="V35" s="5"/>
     </row>
     <row r="36" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="145" t="s">
+      <c r="A36" s="97" t="s">
         <v>37</v>
       </c>
-      <c r="B36" s="141" t="s">
+      <c r="B36" s="93" t="s">
         <v>38</v>
       </c>
-      <c r="C36" s="148"/>
-      <c r="D36" s="148"/>
-      <c r="E36" s="148"/>
+      <c r="C36" s="100"/>
+      <c r="D36" s="100"/>
+      <c r="E36" s="100"/>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
@@ -28080,15 +28114,15 @@
       <c r="V36" s="5"/>
     </row>
     <row r="37" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="146">
+      <c r="A37" s="98">
         <v>1</v>
       </c>
       <c r="B37" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="149"/>
-      <c r="D37" s="149"/>
-      <c r="E37" s="149"/>
+      <c r="C37" s="101"/>
+      <c r="D37" s="101"/>
+      <c r="E37" s="101"/>
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
@@ -28108,13 +28142,13 @@
       <c r="V37" s="5"/>
     </row>
     <row r="38" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="146">
+      <c r="A38" s="98">
         <v>2</v>
       </c>
       <c r="B38" s="12"/>
-      <c r="C38" s="149"/>
-      <c r="D38" s="149"/>
-      <c r="E38" s="149"/>
+      <c r="C38" s="101"/>
+      <c r="D38" s="101"/>
+      <c r="E38" s="101"/>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
       <c r="H38" s="5"/>
@@ -28134,13 +28168,13 @@
       <c r="V38" s="5"/>
     </row>
     <row r="39" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="146" t="s">
+      <c r="A39" s="98" t="s">
         <v>39</v>
       </c>
       <c r="B39" s="12"/>
-      <c r="C39" s="149"/>
-      <c r="D39" s="149"/>
-      <c r="E39" s="149"/>
+      <c r="C39" s="101"/>
+      <c r="D39" s="101"/>
+      <c r="E39" s="101"/>
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5"/>
@@ -28160,15 +28194,15 @@
       <c r="V39" s="5"/>
     </row>
     <row r="40" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="145" t="s">
+      <c r="A40" s="97" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="141" t="s">
+      <c r="B40" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="C40" s="148"/>
-      <c r="D40" s="148"/>
-      <c r="E40" s="148"/>
+      <c r="C40" s="100"/>
+      <c r="D40" s="100"/>
+      <c r="E40" s="100"/>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5"/>
@@ -28188,15 +28222,15 @@
       <c r="V40" s="5"/>
     </row>
     <row r="41" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="146">
+      <c r="A41" s="98">
         <v>1</v>
       </c>
       <c r="B41" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C41" s="149"/>
-      <c r="D41" s="149"/>
-      <c r="E41" s="149"/>
+      <c r="C41" s="101"/>
+      <c r="D41" s="101"/>
+      <c r="E41" s="101"/>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
@@ -28216,13 +28250,13 @@
       <c r="V41" s="5"/>
     </row>
     <row r="42" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="146">
+      <c r="A42" s="98">
         <v>2</v>
       </c>
       <c r="B42" s="12"/>
-      <c r="C42" s="149"/>
-      <c r="D42" s="149"/>
-      <c r="E42" s="149"/>
+      <c r="C42" s="101"/>
+      <c r="D42" s="101"/>
+      <c r="E42" s="101"/>
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
       <c r="H42" s="5"/>
@@ -28242,13 +28276,13 @@
       <c r="V42" s="5"/>
     </row>
     <row r="43" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="146" t="s">
+      <c r="A43" s="98" t="s">
         <v>39</v>
       </c>
       <c r="B43" s="12"/>
-      <c r="C43" s="149"/>
-      <c r="D43" s="149"/>
-      <c r="E43" s="149"/>
+      <c r="C43" s="101"/>
+      <c r="D43" s="101"/>
+      <c r="E43" s="101"/>
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
       <c r="H43" s="5"/>
@@ -28270,9 +28304,9 @@
     <row r="44" spans="1:22" s="79" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="76"/>
       <c r="B44" s="84"/>
-      <c r="C44" s="150"/>
-      <c r="D44" s="150"/>
-      <c r="E44" s="150"/>
+      <c r="C44" s="102"/>
+      <c r="D44" s="102"/>
+      <c r="E44" s="102"/>
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5"/>
@@ -28292,13 +28326,13 @@
       <c r="V44" s="5"/>
     </row>
     <row r="45" spans="1:22" s="82" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A45" s="147"/>
+      <c r="A45" s="99"/>
       <c r="B45" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="C45" s="151"/>
-      <c r="D45" s="151"/>
-      <c r="E45" s="151"/>
+      <c r="C45" s="103"/>
+      <c r="D45" s="103"/>
+      <c r="E45" s="103"/>
       <c r="F45" s="80"/>
       <c r="G45" s="80"/>
       <c r="H45" s="81"/>
@@ -28320,12 +28354,12 @@
     <row r="46" spans="1:22" ht="15.45" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:22" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="85" t="s">
-        <v>156</v>
-      </c>
-      <c r="B47" s="142"/>
-      <c r="C47" s="152"/>
-      <c r="D47" s="155"/>
-      <c r="E47" s="155"/>
+        <v>143</v>
+      </c>
+      <c r="B47" s="94"/>
+      <c r="C47" s="104"/>
+      <c r="D47" s="83"/>
+      <c r="E47" s="83"/>
       <c r="F47" s="83"/>
       <c r="G47" s="83"/>
       <c r="H47" s="83"/>
@@ -28336,12 +28370,12 @@
     </row>
     <row r="48" spans="1:22" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="83" t="s">
-        <v>146</v>
-      </c>
-      <c r="B48" s="143"/>
-      <c r="C48" s="153"/>
-      <c r="D48" s="156"/>
-      <c r="E48" s="156"/>
+        <v>133</v>
+      </c>
+      <c r="B48" s="95"/>
+      <c r="C48" s="105"/>
+      <c r="D48" s="86"/>
+      <c r="E48" s="86"/>
       <c r="F48" s="83"/>
       <c r="G48" s="83"/>
       <c r="H48" s="83"/>
@@ -28349,12 +28383,12 @@
     </row>
     <row r="49" spans="1:12" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="83" t="s">
-        <v>147</v>
-      </c>
-      <c r="B49" s="143"/>
-      <c r="C49" s="153"/>
-      <c r="D49" s="156"/>
-      <c r="E49" s="156"/>
+        <v>134</v>
+      </c>
+      <c r="B49" s="95"/>
+      <c r="C49" s="105"/>
+      <c r="D49" s="86"/>
+      <c r="E49" s="86"/>
       <c r="F49" s="83"/>
       <c r="G49" s="83"/>
       <c r="H49" s="83"/>
@@ -28365,12 +28399,12 @@
     </row>
     <row r="50" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="83" t="s">
-        <v>148</v>
-      </c>
-      <c r="B50" s="143"/>
-      <c r="C50" s="153"/>
-      <c r="D50" s="156"/>
-      <c r="E50" s="156"/>
+        <v>135</v>
+      </c>
+      <c r="B50" s="95"/>
+      <c r="C50" s="105"/>
+      <c r="D50" s="86"/>
+      <c r="E50" s="86"/>
       <c r="F50" s="83"/>
       <c r="G50" s="83"/>
       <c r="H50" s="83"/>
@@ -28381,12 +28415,12 @@
     </row>
     <row r="51" spans="1:12" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="83" t="s">
-        <v>149</v>
-      </c>
-      <c r="B51" s="143"/>
-      <c r="C51" s="153"/>
-      <c r="D51" s="156"/>
-      <c r="E51" s="156"/>
+        <v>136</v>
+      </c>
+      <c r="B51" s="95"/>
+      <c r="C51" s="105"/>
+      <c r="D51" s="86"/>
+      <c r="E51" s="86"/>
       <c r="F51" s="83"/>
       <c r="G51" s="83"/>
       <c r="H51" s="83"/>
@@ -28397,12 +28431,12 @@
     </row>
     <row r="52" spans="1:12" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="83" t="s">
-        <v>150</v>
-      </c>
-      <c r="B52" s="143"/>
-      <c r="C52" s="153"/>
-      <c r="D52" s="156"/>
-      <c r="E52" s="156"/>
+        <v>137</v>
+      </c>
+      <c r="B52" s="95"/>
+      <c r="C52" s="105"/>
+      <c r="D52" s="86"/>
+      <c r="E52" s="86"/>
       <c r="F52" s="83"/>
       <c r="G52" s="83"/>
       <c r="H52" s="83"/>
@@ -28413,12 +28447,12 @@
     </row>
     <row r="53" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A53" s="83" t="s">
-        <v>151</v>
-      </c>
-      <c r="B53" s="143"/>
-      <c r="C53" s="153"/>
-      <c r="D53" s="156"/>
-      <c r="E53" s="156"/>
+        <v>138</v>
+      </c>
+      <c r="B53" s="95"/>
+      <c r="C53" s="105"/>
+      <c r="D53" s="86"/>
+      <c r="E53" s="86"/>
       <c r="F53" s="83"/>
       <c r="G53" s="83"/>
       <c r="H53" s="83"/>
@@ -28426,12 +28460,12 @@
     </row>
     <row r="54" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A54" s="83" t="s">
-        <v>152</v>
-      </c>
-      <c r="B54" s="143"/>
-      <c r="C54" s="153"/>
-      <c r="D54" s="156"/>
-      <c r="E54" s="156"/>
+        <v>139</v>
+      </c>
+      <c r="B54" s="95"/>
+      <c r="C54" s="105"/>
+      <c r="D54" s="86"/>
+      <c r="E54" s="86"/>
       <c r="F54" s="83"/>
       <c r="G54" s="83"/>
       <c r="H54" s="83"/>
@@ -28439,12 +28473,12 @@
     </row>
     <row r="55" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A55" s="83" t="s">
-        <v>153</v>
-      </c>
-      <c r="B55" s="143"/>
-      <c r="C55" s="153"/>
-      <c r="D55" s="156"/>
-      <c r="E55" s="156"/>
+        <v>140</v>
+      </c>
+      <c r="B55" s="95"/>
+      <c r="C55" s="105"/>
+      <c r="D55" s="86"/>
+      <c r="E55" s="86"/>
       <c r="F55" s="83"/>
       <c r="G55" s="83"/>
       <c r="H55" s="83"/>
@@ -28452,132 +28486,132 @@
     </row>
     <row r="56" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A56" s="86" t="s">
-        <v>154</v>
-      </c>
-      <c r="B56" s="143"/>
-      <c r="C56" s="153"/>
-      <c r="D56" s="156"/>
-      <c r="E56" s="156"/>
+        <v>141</v>
+      </c>
+      <c r="B56" s="95"/>
+      <c r="C56" s="105"/>
+      <c r="D56" s="86"/>
+      <c r="E56" s="86"/>
     </row>
     <row r="57" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A57" s="86" t="s">
-        <v>155</v>
-      </c>
-      <c r="B57" s="143"/>
-      <c r="C57" s="153"/>
-      <c r="D57" s="156"/>
-      <c r="E57" s="156"/>
+        <v>142</v>
+      </c>
+      <c r="B57" s="95"/>
+      <c r="C57" s="105"/>
+      <c r="D57" s="86"/>
+      <c r="E57" s="86"/>
     </row>
     <row r="58" spans="1:12" ht="18" x14ac:dyDescent="0.3">
       <c r="A58" s="85" t="s">
-        <v>174</v>
-      </c>
-      <c r="B58" s="142"/>
-      <c r="C58" s="152"/>
-      <c r="D58" s="155"/>
-      <c r="E58" s="155"/>
+        <v>161</v>
+      </c>
+      <c r="B58" s="94"/>
+      <c r="C58" s="104"/>
+      <c r="D58" s="83"/>
+      <c r="E58" s="83"/>
       <c r="F58" s="83"/>
       <c r="G58" s="83"/>
       <c r="H58" s="83"/>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
     </row>
     <row r="61" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>173</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -28621,32 +28655,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="110" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
     </row>
     <row r="2" spans="1:19" ht="13.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="98" t="s">
-        <v>110</v>
-      </c>
-      <c r="B2" s="98"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
+      <c r="A2" s="118" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" s="118"/>
+      <c r="C2" s="118"/>
+      <c r="D2" s="118"/>
+      <c r="E2" s="118"/>
+      <c r="F2" s="118"/>
+      <c r="G2" s="118"/>
+      <c r="H2" s="118"/>
+      <c r="I2" s="118"/>
+      <c r="J2" s="118"/>
       <c r="K2" s="30"/>
       <c r="L2" s="30"/>
       <c r="M2" s="30"/>
@@ -28658,16 +28692,16 @@
       <c r="S2" s="30"/>
     </row>
     <row r="3" spans="1:19" ht="13.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="129"/>
-      <c r="B3" s="129"/>
-      <c r="C3" s="129"/>
-      <c r="D3" s="129"/>
-      <c r="E3" s="129"/>
-      <c r="F3" s="129"/>
-      <c r="G3" s="129"/>
-      <c r="H3" s="129"/>
-      <c r="I3" s="129"/>
-      <c r="J3" s="129"/>
+      <c r="A3" s="156"/>
+      <c r="B3" s="156"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="156"/>
+      <c r="F3" s="156"/>
+      <c r="G3" s="156"/>
+      <c r="H3" s="156"/>
+      <c r="I3" s="156"/>
+      <c r="J3" s="156"/>
       <c r="K3" s="30"/>
       <c r="L3" s="30"/>
       <c r="M3" s="30"/>
@@ -28686,11 +28720,11 @@
       <c r="E4" s="32"/>
       <c r="F4" s="30"/>
       <c r="G4" s="32"/>
-      <c r="H4" s="99" t="s">
-        <v>111</v>
-      </c>
-      <c r="I4" s="99"/>
-      <c r="J4" s="99"/>
+      <c r="H4" s="119" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="119"/>
+      <c r="J4" s="119"/>
       <c r="K4" s="30"/>
       <c r="L4" s="30"/>
       <c r="M4" s="30"/>
@@ -28702,28 +28736,28 @@
       <c r="S4" s="30"/>
     </row>
     <row r="5" spans="1:19" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="100" t="s">
-        <v>112</v>
-      </c>
-      <c r="B5" s="102" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="103" t="s">
-        <v>114</v>
-      </c>
-      <c r="D5" s="104"/>
-      <c r="E5" s="103" t="s">
-        <v>115</v>
-      </c>
-      <c r="F5" s="104"/>
-      <c r="G5" s="103" t="s">
+      <c r="A5" s="120" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="122" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="123" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="124"/>
+      <c r="E5" s="123" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" s="124"/>
+      <c r="G5" s="123" t="s">
         <v>66</v>
       </c>
-      <c r="H5" s="105"/>
-      <c r="I5" s="103" t="s">
+      <c r="H5" s="125"/>
+      <c r="I5" s="123" t="s">
         <v>67</v>
       </c>
-      <c r="J5" s="106"/>
+      <c r="J5" s="126"/>
       <c r="K5" s="30"/>
       <c r="L5" s="30"/>
       <c r="M5" s="30"/>
@@ -28735,8 +28769,8 @@
       <c r="S5" s="30"/>
     </row>
     <row r="6" spans="1:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="101"/>
-      <c r="B6" s="101"/>
+      <c r="A6" s="121"/>
+      <c r="B6" s="121"/>
       <c r="C6" s="33" t="s">
         <v>56</v>
       </c>
@@ -28797,10 +28831,10 @@
         <v>6</v>
       </c>
       <c r="I7" s="35" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="J7" s="35" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="K7" s="36"/>
       <c r="L7" s="36"/>
@@ -29259,16 +29293,16 @@
       <c r="S28" s="30"/>
     </row>
     <row r="29" spans="1:19" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="94"/>
-      <c r="F29" s="94"/>
-      <c r="G29" s="94"/>
-      <c r="H29" s="94"/>
-      <c r="I29" s="94"/>
-      <c r="J29" s="94"/>
+      <c r="A29" s="127"/>
+      <c r="B29" s="127"/>
+      <c r="C29" s="127"/>
+      <c r="D29" s="127"/>
+      <c r="E29" s="127"/>
+      <c r="F29" s="127"/>
+      <c r="G29" s="127"/>
+      <c r="H29" s="127"/>
+      <c r="I29" s="127"/>
+      <c r="J29" s="127"/>
       <c r="K29" s="72"/>
       <c r="L29" s="72"/>
       <c r="M29" s="72"/>
@@ -29287,9 +29321,9 @@
       <c r="E30" s="73"/>
       <c r="F30" s="72"/>
       <c r="G30" s="73"/>
-      <c r="H30" s="95"/>
-      <c r="I30" s="95"/>
-      <c r="J30" s="96"/>
+      <c r="H30" s="128"/>
+      <c r="I30" s="128"/>
+      <c r="J30" s="129"/>
       <c r="K30" s="72"/>
       <c r="L30" s="72"/>
       <c r="M30" s="72"/>
@@ -29302,14 +29336,14 @@
     </row>
     <row r="31" spans="1:19" ht="13.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="22"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="96"/>
-      <c r="E31" s="96"/>
-      <c r="F31" s="96"/>
-      <c r="G31" s="96"/>
-      <c r="H31" s="97"/>
-      <c r="I31" s="97"/>
-      <c r="J31" s="96"/>
+      <c r="C31" s="130"/>
+      <c r="D31" s="129"/>
+      <c r="E31" s="129"/>
+      <c r="F31" s="129"/>
+      <c r="G31" s="129"/>
+      <c r="H31" s="130"/>
+      <c r="I31" s="130"/>
+      <c r="J31" s="129"/>
       <c r="K31" s="22"/>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -29428,14 +29462,14 @@
     <row r="37" spans="1:19" s="75" customFormat="1" ht="13.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="29"/>
       <c r="B37" s="29"/>
-      <c r="C37" s="98"/>
-      <c r="D37" s="98"/>
-      <c r="E37" s="98"/>
-      <c r="F37" s="98"/>
-      <c r="G37" s="98"/>
-      <c r="H37" s="98"/>
-      <c r="I37" s="98"/>
-      <c r="J37" s="98"/>
+      <c r="C37" s="118"/>
+      <c r="D37" s="118"/>
+      <c r="E37" s="118"/>
+      <c r="F37" s="118"/>
+      <c r="G37" s="118"/>
+      <c r="H37" s="118"/>
+      <c r="I37" s="118"/>
+      <c r="J37" s="118"/>
       <c r="K37" s="74"/>
       <c r="L37" s="74"/>
       <c r="M37" s="74"/>
@@ -49790,87 +49824,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="C1" s="107" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="107"/>
-      <c r="O1" s="107"/>
-      <c r="P1" s="107"/>
-      <c r="Q1" s="107"/>
-      <c r="R1" s="107"/>
-      <c r="S1" s="107"/>
-      <c r="T1" s="107"/>
-      <c r="U1" s="107"/>
-      <c r="V1" s="107"/>
-      <c r="W1" s="107"/>
+      <c r="C1" s="110" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="110"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="110"/>
+      <c r="S1" s="110"/>
+      <c r="T1" s="110"/>
+      <c r="U1" s="110"/>
+      <c r="V1" s="110"/>
+      <c r="W1" s="110"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="107" t="s">
+      <c r="C2" s="110" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
-      <c r="M2" s="107"/>
-      <c r="N2" s="107"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="107"/>
-      <c r="Q2" s="107"/>
-      <c r="R2" s="107"/>
-      <c r="S2" s="107"/>
-      <c r="T2" s="107"/>
-      <c r="U2" s="107"/>
-      <c r="V2" s="107"/>
-      <c r="W2" s="107"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
+      <c r="L2" s="110"/>
+      <c r="M2" s="110"/>
+      <c r="N2" s="110"/>
+      <c r="O2" s="110"/>
+      <c r="P2" s="110"/>
+      <c r="Q2" s="110"/>
+      <c r="R2" s="110"/>
+      <c r="S2" s="110"/>
+      <c r="T2" s="110"/>
+      <c r="U2" s="110"/>
+      <c r="V2" s="110"/>
+      <c r="W2" s="110"/>
     </row>
     <row r="3" spans="1:23" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
-      <c r="P3" s="93"/>
-      <c r="Q3" s="93"/>
-      <c r="R3" s="93"/>
-      <c r="S3" s="93"/>
-      <c r="T3" s="93"/>
-      <c r="U3" s="93"/>
-      <c r="V3" s="93"/>
-      <c r="W3" s="93"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115"/>
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="115"/>
+      <c r="S3" s="115"/>
+      <c r="T3" s="115"/>
+      <c r="U3" s="115"/>
+      <c r="V3" s="115"/>
+      <c r="W3" s="115"/>
     </row>
     <row r="4" spans="1:23" s="15" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="C4" s="16"/>
@@ -49890,106 +49924,106 @@
       <c r="W5" s="21"/>
     </row>
     <row r="6" spans="1:23" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="91" t="s">
+      <c r="A6" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="91" t="s">
+      <c r="B6" s="111" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="123" t="s">
+      <c r="C6" s="143" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="91" t="s">
+      <c r="D6" s="111" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="91" t="s">
+      <c r="E6" s="111" t="s">
         <v>102</v>
       </c>
-      <c r="F6" s="91" t="s">
+      <c r="F6" s="111" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="91" t="s">
+      <c r="H6" s="111" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="91" t="s">
+      <c r="I6" s="111" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="91" t="s">
+      <c r="J6" s="111" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="91" t="s">
+      <c r="K6" s="111" t="s">
         <v>53</v>
       </c>
-      <c r="L6" s="91" t="s">
+      <c r="L6" s="111" t="s">
         <v>55</v>
       </c>
-      <c r="M6" s="91" t="s">
+      <c r="M6" s="111" t="s">
         <v>13</v>
       </c>
-      <c r="N6" s="91"/>
-      <c r="O6" s="91"/>
-      <c r="P6" s="91"/>
-      <c r="Q6" s="113" t="s">
+      <c r="N6" s="111"/>
+      <c r="O6" s="111"/>
+      <c r="P6" s="111"/>
+      <c r="Q6" s="112" t="s">
         <v>16</v>
       </c>
-      <c r="R6" s="114"/>
-      <c r="S6" s="114"/>
-      <c r="T6" s="114"/>
-      <c r="U6" s="114"/>
-      <c r="V6" s="115"/>
-      <c r="W6" s="91" t="s">
+      <c r="R6" s="113"/>
+      <c r="S6" s="113"/>
+      <c r="T6" s="113"/>
+      <c r="U6" s="113"/>
+      <c r="V6" s="114"/>
+      <c r="W6" s="111" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:23" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="91"/>
-      <c r="B7" s="91"/>
-      <c r="C7" s="124"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
-      <c r="I7" s="91"/>
-      <c r="J7" s="91"/>
-      <c r="K7" s="91"/>
-      <c r="L7" s="91"/>
-      <c r="M7" s="91" t="s">
+      <c r="A7" s="111"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="144"/>
+      <c r="D7" s="111"/>
+      <c r="E7" s="111"/>
+      <c r="F7" s="111"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="111"/>
+      <c r="I7" s="111"/>
+      <c r="J7" s="111"/>
+      <c r="K7" s="111"/>
+      <c r="L7" s="111"/>
+      <c r="M7" s="111" t="s">
         <v>9</v>
       </c>
-      <c r="N7" s="91"/>
-      <c r="O7" s="91" t="s">
+      <c r="N7" s="111"/>
+      <c r="O7" s="111" t="s">
         <v>12</v>
       </c>
-      <c r="P7" s="91"/>
-      <c r="Q7" s="91" t="s">
+      <c r="P7" s="111"/>
+      <c r="Q7" s="111" t="s">
         <v>14</v>
       </c>
-      <c r="R7" s="91"/>
-      <c r="S7" s="91"/>
-      <c r="T7" s="91" t="s">
+      <c r="R7" s="111"/>
+      <c r="S7" s="111"/>
+      <c r="T7" s="111" t="s">
         <v>15</v>
       </c>
-      <c r="U7" s="91"/>
-      <c r="V7" s="91"/>
-      <c r="W7" s="91"/>
+      <c r="U7" s="111"/>
+      <c r="V7" s="111"/>
+      <c r="W7" s="111"/>
     </row>
     <row r="8" spans="1:23" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="91"/>
-      <c r="B8" s="91"/>
-      <c r="C8" s="125"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
-      <c r="K8" s="91"/>
-      <c r="L8" s="91"/>
+      <c r="A8" s="111"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="145"/>
+      <c r="D8" s="111"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="111"/>
+      <c r="G8" s="111"/>
+      <c r="H8" s="111"/>
+      <c r="I8" s="111"/>
+      <c r="J8" s="111"/>
+      <c r="K8" s="111"/>
+      <c r="L8" s="111"/>
       <c r="M8" s="7" t="s">
         <v>10</v>
       </c>
@@ -50020,7 +50054,7 @@
       <c r="V8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="W8" s="91"/>
+      <c r="W8" s="111"/>
     </row>
     <row r="9" spans="1:23" s="10" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
@@ -50667,33 +50701,43 @@
       <c r="W30" s="12"/>
     </row>
     <row r="31" spans="1:23" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="111" t="s">
+      <c r="B31" s="116" t="s">
         <v>92</v>
       </c>
-      <c r="C31" s="112"/>
-      <c r="D31" s="112"/>
-      <c r="E31" s="112"/>
-      <c r="F31" s="112"/>
-      <c r="G31" s="112"/>
-      <c r="H31" s="112"/>
-      <c r="I31" s="112"/>
-      <c r="J31" s="112"/>
-      <c r="K31" s="112"/>
-      <c r="L31" s="112"/>
-      <c r="M31" s="112"/>
-      <c r="N31" s="112"/>
-      <c r="O31" s="112"/>
-      <c r="P31" s="112"/>
-      <c r="Q31" s="112"/>
-      <c r="R31" s="112"/>
-      <c r="S31" s="112"/>
-      <c r="T31" s="112"/>
-      <c r="U31" s="112"/>
-      <c r="V31" s="112"/>
-      <c r="W31" s="112"/>
+      <c r="C31" s="117"/>
+      <c r="D31" s="117"/>
+      <c r="E31" s="117"/>
+      <c r="F31" s="117"/>
+      <c r="G31" s="117"/>
+      <c r="H31" s="117"/>
+      <c r="I31" s="117"/>
+      <c r="J31" s="117"/>
+      <c r="K31" s="117"/>
+      <c r="L31" s="117"/>
+      <c r="M31" s="117"/>
+      <c r="N31" s="117"/>
+      <c r="O31" s="117"/>
+      <c r="P31" s="117"/>
+      <c r="Q31" s="117"/>
+      <c r="R31" s="117"/>
+      <c r="S31" s="117"/>
+      <c r="T31" s="117"/>
+      <c r="U31" s="117"/>
+      <c r="V31" s="117"/>
+      <c r="W31" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="C1:W1"/>
+    <mergeCell ref="C2:W2"/>
+    <mergeCell ref="C3:W3"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="G6:G8"/>
     <mergeCell ref="B31:W31"/>
     <mergeCell ref="Q6:V6"/>
     <mergeCell ref="W6:W8"/>
@@ -50707,16 +50751,6 @@
     <mergeCell ref="K6:K8"/>
     <mergeCell ref="L6:L8"/>
     <mergeCell ref="M6:P6"/>
-    <mergeCell ref="C1:W1"/>
-    <mergeCell ref="C2:W2"/>
-    <mergeCell ref="C3:W3"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="G6:G8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="55" orientation="landscape" r:id="rId1"/>
@@ -50739,72 +50773,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="110" t="s">
         <v>76</v>
       </c>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="107"/>
-      <c r="O1" s="107"/>
-      <c r="P1" s="107"/>
-      <c r="Q1" s="107"/>
-      <c r="R1" s="107"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="110"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="110"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="107" t="s">
+      <c r="C2" s="110" t="s">
         <v>78</v>
       </c>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
-      <c r="M2" s="107"/>
-      <c r="N2" s="107"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="107"/>
-      <c r="Q2" s="107"/>
-      <c r="R2" s="107"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="110"/>
+      <c r="I2" s="110"/>
+      <c r="J2" s="110"/>
+      <c r="K2" s="110"/>
+      <c r="L2" s="110"/>
+      <c r="M2" s="110"/>
+      <c r="N2" s="110"/>
+      <c r="O2" s="110"/>
+      <c r="P2" s="110"/>
+      <c r="Q2" s="110"/>
+      <c r="R2" s="110"/>
     </row>
     <row r="3" spans="1:19" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="93" t="s">
+      <c r="C3" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
-      <c r="P3" s="93"/>
-      <c r="Q3" s="93"/>
-      <c r="R3" s="93"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115"/>
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="115"/>
     </row>
     <row r="4" spans="1:19" s="15" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="C4" s="16"/>
@@ -50813,109 +50847,109 @@
       <c r="F4" s="16"/>
     </row>
     <row r="6" spans="1:19" s="1" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="91" t="s">
+      <c r="A6" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="91" t="s">
+      <c r="B6" s="111" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="91" t="s">
+      <c r="C6" s="111" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="91" t="s">
+      <c r="D6" s="111" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="91" t="s">
+      <c r="E6" s="111" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="91" t="s">
+      <c r="F6" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="91" t="s">
+      <c r="H6" s="111" t="s">
         <v>84</v>
       </c>
-      <c r="I6" s="91"/>
-      <c r="J6" s="91"/>
-      <c r="K6" s="113" t="s">
+      <c r="I6" s="111"/>
+      <c r="J6" s="111"/>
+      <c r="K6" s="112" t="s">
         <v>79</v>
       </c>
-      <c r="L6" s="114"/>
-      <c r="M6" s="114"/>
-      <c r="N6" s="114"/>
-      <c r="O6" s="114"/>
-      <c r="P6" s="115"/>
-      <c r="Q6" s="123" t="s">
+      <c r="L6" s="113"/>
+      <c r="M6" s="113"/>
+      <c r="N6" s="113"/>
+      <c r="O6" s="113"/>
+      <c r="P6" s="114"/>
+      <c r="Q6" s="143" t="s">
         <v>83</v>
       </c>
-      <c r="R6" s="91" t="s">
+      <c r="R6" s="111" t="s">
         <v>75</v>
       </c>
-      <c r="S6" s="130"/>
+      <c r="S6" s="157"/>
     </row>
     <row r="7" spans="1:19" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="91"/>
-      <c r="B7" s="91"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91" t="s">
+      <c r="A7" s="111"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="111"/>
+      <c r="D7" s="111"/>
+      <c r="E7" s="111"/>
+      <c r="F7" s="111"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="111" t="s">
         <v>72</v>
       </c>
-      <c r="I7" s="91" t="s">
+      <c r="I7" s="111" t="s">
         <v>74</v>
       </c>
-      <c r="J7" s="91" t="s">
+      <c r="J7" s="111" t="s">
         <v>73</v>
       </c>
-      <c r="K7" s="113" t="s">
+      <c r="K7" s="112" t="s">
         <v>87</v>
       </c>
-      <c r="L7" s="114"/>
-      <c r="M7" s="91" t="s">
+      <c r="L7" s="113"/>
+      <c r="M7" s="111" t="s">
         <v>80</v>
       </c>
-      <c r="N7" s="91" t="s">
+      <c r="N7" s="111" t="s">
         <v>81</v>
       </c>
-      <c r="O7" s="123" t="s">
+      <c r="O7" s="143" t="s">
         <v>82</v>
       </c>
-      <c r="P7" s="123" t="s">
+      <c r="P7" s="143" t="s">
         <v>39</v>
       </c>
-      <c r="Q7" s="124"/>
-      <c r="R7" s="91"/>
-      <c r="S7" s="130"/>
+      <c r="Q7" s="144"/>
+      <c r="R7" s="111"/>
+      <c r="S7" s="157"/>
     </row>
     <row r="8" spans="1:19" ht="89.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="91"/>
-      <c r="B8" s="91"/>
-      <c r="C8" s="91"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
-      <c r="I8" s="91"/>
-      <c r="J8" s="91"/>
+      <c r="A8" s="111"/>
+      <c r="B8" s="111"/>
+      <c r="C8" s="111"/>
+      <c r="D8" s="111"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="111"/>
+      <c r="G8" s="111"/>
+      <c r="H8" s="111"/>
+      <c r="I8" s="111"/>
+      <c r="J8" s="111"/>
       <c r="K8" s="5" t="s">
         <v>88</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="M8" s="91"/>
-      <c r="N8" s="91"/>
-      <c r="O8" s="125"/>
-      <c r="P8" s="125"/>
-      <c r="Q8" s="125"/>
-      <c r="R8" s="91"/>
-      <c r="S8" s="130"/>
+      <c r="M8" s="111"/>
+      <c r="N8" s="111"/>
+      <c r="O8" s="145"/>
+      <c r="P8" s="145"/>
+      <c r="Q8" s="145"/>
+      <c r="R8" s="111"/>
+      <c r="S8" s="157"/>
     </row>
     <row r="9" spans="1:19" s="10" customFormat="1" ht="10.199999999999999" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
@@ -51442,43 +51476,29 @@
       <c r="R30" s="12"/>
     </row>
     <row r="31" spans="1:18" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="111" t="s">
+      <c r="A31" s="116" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="111"/>
-      <c r="C31" s="111"/>
-      <c r="D31" s="111"/>
-      <c r="E31" s="111"/>
-      <c r="F31" s="111"/>
-      <c r="G31" s="111"/>
-      <c r="H31" s="111"/>
-      <c r="I31" s="111"/>
-      <c r="J31" s="111"/>
-      <c r="K31" s="111"/>
-      <c r="L31" s="111"/>
-      <c r="M31" s="111"/>
-      <c r="N31" s="111"/>
-      <c r="O31" s="111"/>
-      <c r="P31" s="111"/>
-      <c r="Q31" s="111"/>
-      <c r="R31" s="111"/>
+      <c r="B31" s="116"/>
+      <c r="C31" s="116"/>
+      <c r="D31" s="116"/>
+      <c r="E31" s="116"/>
+      <c r="F31" s="116"/>
+      <c r="G31" s="116"/>
+      <c r="H31" s="116"/>
+      <c r="I31" s="116"/>
+      <c r="J31" s="116"/>
+      <c r="K31" s="116"/>
+      <c r="L31" s="116"/>
+      <c r="M31" s="116"/>
+      <c r="N31" s="116"/>
+      <c r="O31" s="116"/>
+      <c r="P31" s="116"/>
+      <c r="Q31" s="116"/>
+      <c r="R31" s="116"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A31:R31"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="K6:P6"/>
-    <mergeCell ref="Q6:Q8"/>
-    <mergeCell ref="R6:R8"/>
-    <mergeCell ref="S6:S8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="P7:P8"/>
     <mergeCell ref="C1:R1"/>
     <mergeCell ref="C2:R2"/>
     <mergeCell ref="C3:R3"/>
@@ -51489,6 +51509,20 @@
     <mergeCell ref="E6:E8"/>
     <mergeCell ref="F6:F8"/>
     <mergeCell ref="G6:G8"/>
+    <mergeCell ref="S6:S8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="P7:P8"/>
+    <mergeCell ref="A31:R31"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="K6:P6"/>
+    <mergeCell ref="Q6:Q8"/>
+    <mergeCell ref="R6:R8"/>
   </mergeCells>
   <pageMargins left="0.2" right="0.2" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="68" orientation="landscape" r:id="rId1"/>

</xml_diff>